<commit_message>
Enhance stringing plan functionality and integrate new data handling
- Added new functions to retrieve stringing responsibilities and completion keys in `app.py`.
- Updated the `create_app` function to include new providers for stringing plan data.
- Refactored the `pipeline_runner.py` to compile stringing micro plans and handle output paths.
- Improved error handling and data normalization in the `data_loader.py` for stringing artifacts.
- Updated binary files to reflect recent changes in stringing data processing and outputs.
</commit_message>
<xml_diff>
--- a/Raw Data/Micro Plans/November 2025/Micro Plan - TA-413 Nov'25.xlsx
+++ b/Raw Data/Micro Plans/November 2025/Micro Plan - TA-413 Nov'25.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://rpgnet-my.sharepoint.com/personal/kumarsan50_kecrpg_com/Documents/Miscellaneous/Sourabh Das/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kaushikb\Documents\Work\Git\Office-work-\Raw Data\Micro Plans\November 2025\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="294" documentId="13_ncr:1_{42ADFFED-B495-4418-A6FB-72AC580E0EC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4E4DF607-1C74-45BD-A30A-45CCCB811832}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F4D9C61-9FC6-4092-B033-11C8089F33F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="757" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="757" firstSheet="2" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="FDN-June25" sheetId="1" state="hidden" r:id="rId1"/>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="418" uniqueCount="222">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="447" uniqueCount="231">
   <si>
     <t>Project Code</t>
   </si>
@@ -657,18 +657,6 @@
     <t>Datewise Stringing planning for the month of November 2025</t>
   </si>
   <si>
-    <t>Sr no</t>
-  </si>
-  <si>
-    <t>Section Name</t>
-  </si>
-  <si>
-    <t>Tower Erection  Status</t>
-  </si>
-  <si>
-    <t>Tower in section</t>
-  </si>
-  <si>
     <t>Insulator Hoisting</t>
   </si>
   <si>
@@ -678,43 +666,82 @@
     <t>Paying Out Completed</t>
   </si>
   <si>
-    <t>Final sag complete</t>
-  </si>
-  <si>
-    <t>AP-6 - AP-7/0</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Complete </t>
-  </si>
-  <si>
     <t>Rahim Khan</t>
   </si>
   <si>
-    <t>AP-5 - AP-5A/0</t>
-  </si>
-  <si>
-    <t>AP-5A/0 - AP-6</t>
-  </si>
-  <si>
-    <t>AP-32A/0 - AP-33/0</t>
-  </si>
-  <si>
     <t>Tanjira Bibi</t>
   </si>
   <si>
-    <t>AP-32/0 - AP-32A/0</t>
-  </si>
-  <si>
-    <t>AP-33/0 - AP-34/0</t>
-  </si>
-  <si>
-    <t>Total length (KM)</t>
-  </si>
-  <si>
     <t xml:space="preserve">Micro Plan - Stringing </t>
   </si>
   <si>
-    <t>Section Length Miter</t>
+    <t>S. No.</t>
+  </si>
+  <si>
+    <t>From AP</t>
+  </si>
+  <si>
+    <t>To AP</t>
+  </si>
+  <si>
+    <t>Span (m)</t>
+  </si>
+  <si>
+    <t>Tower Erection Status</t>
+  </si>
+  <si>
+    <t>Towers in Section</t>
+  </si>
+  <si>
+    <t>Final Sag Complete</t>
+  </si>
+  <si>
+    <t>Method</t>
+  </si>
+  <si>
+    <t>Gang Strength</t>
+  </si>
+  <si>
+    <t>Complete</t>
+  </si>
+  <si>
+    <t>D1</t>
+  </si>
+  <si>
+    <t>D2</t>
+  </si>
+  <si>
+    <t>A</t>
+  </si>
+  <si>
+    <t>B</t>
+  </si>
+  <si>
+    <t>C</t>
+  </si>
+  <si>
+    <t>D</t>
+  </si>
+  <si>
+    <t>E</t>
+  </si>
+  <si>
+    <t>5A/0</t>
+  </si>
+  <si>
+    <t>32A/0</t>
+  </si>
+  <si>
+    <t>33/0</t>
+  </si>
+  <si>
+    <t>32/0</t>
+  </si>
+  <si>
+    <t>34/0</t>
+  </si>
+  <si>
+    <t>7/0</t>
   </si>
 </sst>
 </file>
@@ -722,17 +749,17 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="9">
-    <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="164" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="165" formatCode="[$-409]d\-mmm\-yy;@"/>
-    <numFmt numFmtId="166" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
-    <numFmt numFmtId="167" formatCode="[$-409]d/mmm/yy;@"/>
-    <numFmt numFmtId="168" formatCode="0.0"/>
-    <numFmt numFmtId="169" formatCode="#,##0.000"/>
-    <numFmt numFmtId="170" formatCode="0.000"/>
-    <numFmt numFmtId="171" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="164" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="165" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="166" formatCode="[$-409]d\-mmm\-yy;@"/>
+    <numFmt numFmtId="167" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
+    <numFmt numFmtId="168" formatCode="[$-409]d/mmm/yy;@"/>
+    <numFmt numFmtId="169" formatCode="0.0"/>
+    <numFmt numFmtId="170" formatCode="#,##0.000"/>
+    <numFmt numFmtId="171" formatCode="0.000"/>
+    <numFmt numFmtId="172" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
-  <fonts count="35" x14ac:knownFonts="1">
+  <fonts count="34" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -943,12 +970,6 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
       <sz val="12"/>
       <color indexed="8"/>
       <name val="Verdana"/>
@@ -974,7 +995,7 @@
       <family val="1"/>
     </font>
   </fonts>
-  <fills count="13">
+  <fills count="12">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1040,14 +1061,8 @@
         <fgColor rgb="FFFFFFCC"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.79998168889431442"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="30">
+  <borders count="25">
     <border>
       <left/>
       <right/>
@@ -1294,36 +1309,6 @@
       <diagonal/>
     </border>
     <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left/>
       <right/>
       <top style="medium">
@@ -1363,19 +1348,6 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
       <left style="medium">
         <color indexed="64"/>
       </left>
@@ -1409,30 +1381,6 @@
         <color indexed="64"/>
       </right>
       <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top/>
       <bottom style="medium">
         <color indexed="64"/>
       </bottom>
@@ -1441,14 +1389,14 @@
   </borders>
   <cellStyleXfs count="172">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0"/>
-    <xf numFmtId="167" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="167" fontId="13" fillId="0" borderId="0"/>
+    <xf numFmtId="168" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="168" fontId="13" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="13" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0"/>
@@ -1467,21 +1415,21 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="43" fontId="13" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="43" fontId="13" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="170" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="171" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
@@ -1501,13 +1449,13 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0">
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0">
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0">
@@ -1579,11 +1527,11 @@
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="18" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="11" borderId="15" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
@@ -1626,36 +1574,36 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="34" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="171" fontId="13" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="0"/>
+    <xf numFmtId="164" fontId="33" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="172" fontId="13" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0"/>
-    <xf numFmtId="171" fontId="13" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="172" fontId="13" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0"/>
-    <xf numFmtId="171" fontId="13" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="172" fontId="13" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="13" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="43" fontId="13" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="43" fontId="13" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="43" fontId="34" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="164" fontId="33" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="241">
+  <cellXfs count="228">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -1699,13 +1647,13 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="43" fontId="3" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1714,25 +1662,25 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="3" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1741,31 +1689,31 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="43" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="43" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="10" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="43" fontId="3" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="43" fontId="3" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="43" fontId="3" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1774,13 +1722,13 @@
     <xf numFmtId="17" fontId="3" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="0" fillId="4" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="4" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="10" fillId="4" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="3" fillId="4" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="3" fillId="4" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1795,7 +1743,7 @@
     <xf numFmtId="9" fontId="11" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="9" fontId="11" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
@@ -1810,41 +1758,41 @@
     <xf numFmtId="2" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="3" fillId="5" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="3" fillId="5" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="3" fillId="4" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="3" fillId="4" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="15" fillId="4" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="15" fillId="4" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="17" fillId="6" borderId="14" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="17" fillId="6" borderId="14" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="17" fillId="6" borderId="14" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="166" fontId="17" fillId="6" borderId="14" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
     <xf numFmtId="1" fontId="17" fillId="6" borderId="14" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="17" fillId="6" borderId="14" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="17" fillId="6" borderId="14" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="167" fontId="18" fillId="0" borderId="1" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="168" fontId="18" fillId="0" borderId="1" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="19" fillId="0" borderId="1" xfId="6" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="19" fillId="0" borderId="1" xfId="6" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="18" fillId="0" borderId="1" xfId="6" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="18" fillId="0" borderId="1" xfId="6" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="18" fillId="0" borderId="1" xfId="6" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="18" fillId="0" borderId="1" xfId="6" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="1" xfId="6" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1872,7 +1820,7 @@
     <xf numFmtId="1" fontId="20" fillId="0" borderId="1" xfId="7" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="168" fontId="18" fillId="8" borderId="3" xfId="7" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="169" fontId="18" fillId="8" borderId="3" xfId="7" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
@@ -1885,7 +1833,7 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="43" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1909,16 +1857,16 @@
     <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" quotePrefix="1" applyBorder="1" applyAlignment="1">
@@ -1930,16 +1878,16 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="14" fontId="13" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1951,7 +1899,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="169" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="170" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1990,19 +1938,19 @@
     <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -2011,7 +1959,7 @@
     <xf numFmtId="2" fontId="26" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="170" fontId="26" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="171" fontId="26" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2020,7 +1968,7 @@
     <xf numFmtId="2" fontId="26" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="170" fontId="3" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="171" fontId="3" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
@@ -2062,13 +2010,13 @@
     <xf numFmtId="0" fontId="13" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="170" fontId="23" fillId="10" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="171" fontId="23" fillId="10" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="27" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="11" fillId="10" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="11" fillId="10" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="1" fontId="11" fillId="10" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2107,16 +2055,16 @@
     <xf numFmtId="14" fontId="0" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="10" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="0" fillId="10" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="43" fontId="11" fillId="10" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="11" fillId="10" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="43" fontId="12" fillId="10" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="12" fillId="10" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="43" fontId="11" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="11" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="27" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2161,17 +2109,16 @@
     <xf numFmtId="0" fontId="14" fillId="10" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="170" fontId="29" fillId="10" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="171" fontId="29" fillId="10" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="15" fontId="14" fillId="10" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -2187,19 +2134,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
@@ -2208,27 +2149,30 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="15" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2319,42 +2263,6 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="12" borderId="20" xfId="78" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="12" borderId="1" xfId="78" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="24" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="27" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="18" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="12" borderId="19" xfId="78" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="12" borderId="16" xfId="78" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="12" borderId="28" xfId="78" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="12" borderId="18" xfId="78" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -2366,6 +2274,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="172">
@@ -5916,10 +5827,6 @@
 </externalLink>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -6187,38 +6094,38 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AG34"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="4.140625" style="4" customWidth="1"/>
+    <col min="1" max="1" width="4.1796875" style="4" customWidth="1"/>
     <col min="2" max="3" width="10" style="1" customWidth="1"/>
-    <col min="4" max="4" width="12.5703125" style="4" customWidth="1"/>
-    <col min="5" max="6" width="8.7109375" style="4" customWidth="1"/>
-    <col min="7" max="7" width="22.28515625" style="4" customWidth="1"/>
-    <col min="8" max="8" width="14.28515625" style="1" customWidth="1"/>
-    <col min="9" max="9" width="11.5703125" style="1" customWidth="1"/>
-    <col min="10" max="10" width="12.5703125" style="1" customWidth="1"/>
-    <col min="11" max="11" width="16.140625" style="1" customWidth="1"/>
-    <col min="12" max="12" width="12.140625" style="1" customWidth="1"/>
-    <col min="13" max="13" width="14.85546875" style="1" customWidth="1"/>
-    <col min="14" max="14" width="11.28515625" style="1" customWidth="1"/>
-    <col min="15" max="15" width="12.140625" style="1" customWidth="1"/>
-    <col min="16" max="16" width="17.7109375" style="1" customWidth="1"/>
-    <col min="17" max="17" width="3.140625" style="1" customWidth="1"/>
-    <col min="18" max="18" width="14.5703125" style="1" customWidth="1"/>
-    <col min="19" max="19" width="3.140625" style="1" customWidth="1"/>
-    <col min="20" max="25" width="8.7109375" style="1" customWidth="1"/>
-    <col min="26" max="26" width="3.140625" style="1" customWidth="1"/>
+    <col min="4" max="4" width="12.54296875" style="4" customWidth="1"/>
+    <col min="5" max="6" width="8.7265625" style="4" customWidth="1"/>
+    <col min="7" max="7" width="22.26953125" style="4" customWidth="1"/>
+    <col min="8" max="8" width="14.26953125" style="1" customWidth="1"/>
+    <col min="9" max="9" width="11.54296875" style="1" customWidth="1"/>
+    <col min="10" max="10" width="12.54296875" style="1" customWidth="1"/>
+    <col min="11" max="11" width="16.1796875" style="1" customWidth="1"/>
+    <col min="12" max="12" width="12.1796875" style="1" customWidth="1"/>
+    <col min="13" max="13" width="14.81640625" style="1" customWidth="1"/>
+    <col min="14" max="14" width="11.26953125" style="1" customWidth="1"/>
+    <col min="15" max="15" width="12.1796875" style="1" customWidth="1"/>
+    <col min="16" max="16" width="17.7265625" style="1" customWidth="1"/>
+    <col min="17" max="17" width="3.1796875" style="1" customWidth="1"/>
+    <col min="18" max="18" width="14.54296875" style="1" customWidth="1"/>
+    <col min="19" max="19" width="3.1796875" style="1" customWidth="1"/>
+    <col min="20" max="25" width="8.7265625" style="1" customWidth="1"/>
+    <col min="26" max="26" width="3.1796875" style="1" customWidth="1"/>
     <col min="27" max="27" width="15" style="1" customWidth="1"/>
-    <col min="28" max="28" width="15.5703125" style="1" customWidth="1"/>
-    <col min="29" max="29" width="17.140625" style="1" customWidth="1"/>
-    <col min="30" max="30" width="13.85546875" style="1" customWidth="1"/>
-    <col min="31" max="31" width="10.7109375" style="1" customWidth="1"/>
-    <col min="32" max="32" width="15.5703125" style="1" customWidth="1"/>
-    <col min="33" max="33" width="17.140625" style="1" customWidth="1"/>
-    <col min="34" max="16384" width="9.140625" style="1"/>
+    <col min="28" max="28" width="15.54296875" style="1" customWidth="1"/>
+    <col min="29" max="29" width="17.1796875" style="1" customWidth="1"/>
+    <col min="30" max="30" width="13.81640625" style="1" customWidth="1"/>
+    <col min="31" max="31" width="10.7265625" style="1" customWidth="1"/>
+    <col min="32" max="32" width="15.54296875" style="1" customWidth="1"/>
+    <col min="33" max="33" width="17.1796875" style="1" customWidth="1"/>
+    <col min="34" max="16384" width="9.1796875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A1" s="13" t="s">
         <v>0</v>
       </c>
@@ -6226,7 +6133,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A2" s="13" t="s">
         <v>21</v>
       </c>
@@ -6234,11 +6141,11 @@
         <v>49</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A3" s="6"/>
       <c r="D3" s="1"/>
     </row>
-    <row r="4" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:13" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A4" s="13" t="s">
         <v>22</v>
       </c>
@@ -6254,7 +6161,7 @@
       <c r="L4" s="82"/>
       <c r="M4" s="83"/>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A5" s="6"/>
       <c r="D5" s="2" t="s">
         <v>29</v>
@@ -6265,7 +6172,7 @@
       <c r="J5" s="4"/>
       <c r="K5" s="4"/>
     </row>
-    <row r="6" spans="1:13" ht="17.25" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:13" ht="16" x14ac:dyDescent="0.35">
       <c r="A6" s="6"/>
       <c r="D6" s="2" t="s">
         <v>85</v>
@@ -6276,7 +6183,7 @@
       <c r="K6" s="3"/>
       <c r="M6" s="97"/>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A7" s="6"/>
       <c r="D7" s="2" t="s">
         <v>2</v>
@@ -6288,11 +6195,11 @@
       <c r="K7" s="3"/>
       <c r="M7" s="97"/>
     </row>
-    <row r="8" spans="1:13" ht="5.0999999999999996" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:13" ht="5.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A8" s="6"/>
       <c r="D8" s="1"/>
     </row>
-    <row r="9" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A9" s="13" t="s">
         <v>23</v>
       </c>
@@ -6313,13 +6220,13 @@
         <v>20</v>
       </c>
     </row>
-    <row r="10" spans="1:13" ht="5.0999999999999996" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:13" ht="5.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="13"/>
       <c r="D10" s="1"/>
       <c r="E10" s="1"/>
       <c r="F10" s="13"/>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A11" s="13" t="s">
         <v>33</v>
       </c>
@@ -6343,7 +6250,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A12" s="5"/>
       <c r="D12" s="2" t="s">
         <v>25</v>
@@ -6365,7 +6272,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A13" s="5"/>
       <c r="D13" s="2" t="s">
         <v>26</v>
@@ -6387,7 +6294,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A14" s="5"/>
       <c r="D14" s="2" t="s">
         <v>27</v>
@@ -6409,7 +6316,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:13" ht="17.25" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:13" ht="16" x14ac:dyDescent="0.35">
       <c r="A15" s="5"/>
       <c r="D15" s="28" t="s">
         <v>28</v>
@@ -6431,7 +6338,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A16" s="5" t="s">
         <v>51</v>
       </c>
@@ -6455,144 +6362,144 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A17" s="5"/>
       <c r="D17" s="6"/>
       <c r="E17" s="6"/>
       <c r="F17" s="6"/>
     </row>
-    <row r="18" spans="1:33" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="213" t="s">
+    <row r="18" spans="1:33" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A18" s="211" t="s">
         <v>4</v>
       </c>
-      <c r="B18" s="213" t="s">
+      <c r="B18" s="211" t="s">
         <v>5</v>
       </c>
-      <c r="C18" s="209" t="s">
+      <c r="C18" s="207" t="s">
         <v>6</v>
       </c>
-      <c r="D18" s="213" t="s">
+      <c r="D18" s="211" t="s">
         <v>7</v>
       </c>
-      <c r="E18" s="209" t="s">
+      <c r="E18" s="207" t="s">
         <v>16</v>
       </c>
-      <c r="F18" s="209" t="s">
+      <c r="F18" s="207" t="s">
         <v>17</v>
       </c>
-      <c r="G18" s="213" t="s">
+      <c r="G18" s="211" t="s">
         <v>8</v>
       </c>
-      <c r="H18" s="200" t="s">
+      <c r="H18" s="198" t="s">
         <v>18</v>
       </c>
-      <c r="I18" s="200"/>
-      <c r="J18" s="200"/>
-      <c r="K18" s="200"/>
-      <c r="L18" s="200"/>
-      <c r="M18" s="200"/>
-      <c r="N18" s="200"/>
-      <c r="O18" s="200"/>
-      <c r="P18" s="203" t="s">
+      <c r="I18" s="198"/>
+      <c r="J18" s="198"/>
+      <c r="K18" s="198"/>
+      <c r="L18" s="198"/>
+      <c r="M18" s="198"/>
+      <c r="N18" s="198"/>
+      <c r="O18" s="198"/>
+      <c r="P18" s="201" t="s">
         <v>19</v>
       </c>
-      <c r="R18" s="209" t="s">
+      <c r="R18" s="207" t="s">
         <v>36</v>
       </c>
-      <c r="T18" s="204" t="s">
+      <c r="T18" s="202" t="s">
         <v>31</v>
       </c>
-      <c r="U18" s="205"/>
-      <c r="V18" s="205"/>
-      <c r="W18" s="205"/>
-      <c r="X18" s="205"/>
-      <c r="Y18" s="206"/>
-      <c r="AA18" s="204" t="s">
+      <c r="U18" s="203"/>
+      <c r="V18" s="203"/>
+      <c r="W18" s="203"/>
+      <c r="X18" s="203"/>
+      <c r="Y18" s="204"/>
+      <c r="AA18" s="202" t="s">
         <v>30</v>
       </c>
-      <c r="AB18" s="205"/>
-      <c r="AC18" s="205"/>
-      <c r="AD18" s="205"/>
-      <c r="AE18" s="205"/>
-      <c r="AF18" s="206"/>
-      <c r="AG18" s="207" t="s">
+      <c r="AB18" s="203"/>
+      <c r="AC18" s="203"/>
+      <c r="AD18" s="203"/>
+      <c r="AE18" s="203"/>
+      <c r="AF18" s="204"/>
+      <c r="AG18" s="205" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="19" spans="1:33" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="214"/>
-      <c r="B19" s="214"/>
-      <c r="C19" s="211"/>
-      <c r="D19" s="214"/>
-      <c r="E19" s="211"/>
-      <c r="F19" s="211"/>
-      <c r="G19" s="214"/>
-      <c r="H19" s="199" t="s">
+    <row r="19" spans="1:33" ht="21" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A19" s="212"/>
+      <c r="B19" s="212"/>
+      <c r="C19" s="209"/>
+      <c r="D19" s="212"/>
+      <c r="E19" s="209"/>
+      <c r="F19" s="209"/>
+      <c r="G19" s="212"/>
+      <c r="H19" s="197" t="s">
         <v>9</v>
       </c>
-      <c r="I19" s="199"/>
-      <c r="J19" s="199" t="s">
+      <c r="I19" s="197"/>
+      <c r="J19" s="197" t="s">
         <v>12</v>
       </c>
-      <c r="K19" s="199"/>
-      <c r="L19" s="199" t="s">
+      <c r="K19" s="197"/>
+      <c r="L19" s="197" t="s">
         <v>13</v>
       </c>
-      <c r="M19" s="199"/>
-      <c r="N19" s="197" t="s">
+      <c r="M19" s="197"/>
+      <c r="N19" s="195" t="s">
         <v>15</v>
       </c>
-      <c r="O19" s="197" t="s">
+      <c r="O19" s="195" t="s">
         <v>14</v>
       </c>
-      <c r="P19" s="203"/>
-      <c r="R19" s="210"/>
-      <c r="T19" s="201" t="s">
+      <c r="P19" s="201"/>
+      <c r="R19" s="208"/>
+      <c r="T19" s="199" t="s">
         <v>24</v>
       </c>
-      <c r="U19" s="201" t="s">
+      <c r="U19" s="199" t="s">
         <v>25</v>
       </c>
-      <c r="V19" s="201" t="s">
+      <c r="V19" s="199" t="s">
         <v>26</v>
       </c>
-      <c r="W19" s="201" t="s">
+      <c r="W19" s="199" t="s">
         <v>27</v>
       </c>
-      <c r="X19" s="201" t="s">
+      <c r="X19" s="199" t="s">
         <v>28</v>
       </c>
       <c r="Y19" s="43" t="s">
         <v>29</v>
       </c>
-      <c r="AA19" s="201" t="s">
+      <c r="AA19" s="199" t="s">
         <v>24</v>
       </c>
-      <c r="AB19" s="201" t="s">
+      <c r="AB19" s="199" t="s">
         <v>25</v>
       </c>
-      <c r="AC19" s="201" t="s">
+      <c r="AC19" s="199" t="s">
         <v>26</v>
       </c>
-      <c r="AD19" s="201" t="s">
+      <c r="AD19" s="199" t="s">
         <v>27</v>
       </c>
-      <c r="AE19" s="201" t="s">
+      <c r="AE19" s="199" t="s">
         <v>28</v>
       </c>
       <c r="AF19" s="43" t="s">
         <v>29</v>
       </c>
-      <c r="AG19" s="208"/>
-    </row>
-    <row r="20" spans="1:33" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="215"/>
-      <c r="B20" s="214"/>
-      <c r="C20" s="211"/>
-      <c r="D20" s="214"/>
-      <c r="E20" s="212"/>
-      <c r="F20" s="212"/>
-      <c r="G20" s="214"/>
+      <c r="AG19" s="206"/>
+    </row>
+    <row r="20" spans="1:33" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A20" s="213"/>
+      <c r="B20" s="212"/>
+      <c r="C20" s="209"/>
+      <c r="D20" s="212"/>
+      <c r="E20" s="210"/>
+      <c r="F20" s="210"/>
+      <c r="G20" s="212"/>
       <c r="H20" s="93" t="s">
         <v>10</v>
       </c>
@@ -6611,25 +6518,25 @@
       <c r="M20" s="93" t="s">
         <v>11</v>
       </c>
-      <c r="N20" s="198"/>
-      <c r="O20" s="198"/>
+      <c r="N20" s="196"/>
+      <c r="O20" s="196"/>
       <c r="P20" s="44" t="s">
         <v>50</v>
       </c>
       <c r="R20" s="18" t="s">
         <v>37</v>
       </c>
-      <c r="T20" s="202"/>
-      <c r="U20" s="202"/>
-      <c r="V20" s="202"/>
-      <c r="W20" s="202"/>
-      <c r="X20" s="202"/>
+      <c r="T20" s="200"/>
+      <c r="U20" s="200"/>
+      <c r="V20" s="200"/>
+      <c r="W20" s="200"/>
+      <c r="X20" s="200"/>
       <c r="Y20" s="19"/>
-      <c r="AA20" s="202"/>
-      <c r="AB20" s="202"/>
-      <c r="AC20" s="202"/>
-      <c r="AD20" s="202"/>
-      <c r="AE20" s="202"/>
+      <c r="AA20" s="200"/>
+      <c r="AB20" s="200"/>
+      <c r="AC20" s="200"/>
+      <c r="AD20" s="200"/>
+      <c r="AE20" s="200"/>
       <c r="AF20" s="19" t="s">
         <v>50</v>
       </c>
@@ -6637,7 +6544,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="21" spans="1:33" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:33" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A21" s="96">
         <v>1</v>
       </c>
@@ -6729,7 +6636,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:33" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:33" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A22" s="96">
         <v>2</v>
       </c>
@@ -6775,7 +6682,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:33" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:33" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A23" s="96">
         <v>3</v>
       </c>
@@ -6833,7 +6740,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:33" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:33" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A24" s="96">
         <v>4</v>
       </c>
@@ -6891,7 +6798,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:33" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:33" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A25" s="96">
         <v>5</v>
       </c>
@@ -6900,7 +6807,7 @@
       <c r="D25" s="85"/>
       <c r="E25" s="100"/>
       <c r="F25" s="8"/>
-      <c r="G25" s="195"/>
+      <c r="G25" s="193"/>
       <c r="H25" s="98"/>
       <c r="I25" s="98"/>
       <c r="J25" s="98"/>
@@ -6949,7 +6856,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:33" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:33" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A26" s="96">
         <v>6</v>
       </c>
@@ -6958,7 +6865,7 @@
       <c r="D26" s="8"/>
       <c r="E26" s="101"/>
       <c r="F26" s="96"/>
-      <c r="G26" s="196"/>
+      <c r="G26" s="194"/>
       <c r="H26" s="98"/>
       <c r="I26" s="98"/>
       <c r="J26" s="98"/>
@@ -7007,7 +6914,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:33" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:33" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A27" s="96">
         <v>7</v>
       </c>
@@ -7065,7 +6972,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:33" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:33" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A28" s="96"/>
       <c r="B28" s="102"/>
       <c r="C28" s="102"/>
@@ -7121,7 +7028,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:33" ht="20.100000000000001" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:33" ht="20.149999999999999" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A29" s="11"/>
       <c r="B29" s="91"/>
       <c r="C29" s="92"/>
@@ -7177,7 +7084,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:33" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:33" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A30" s="9"/>
       <c r="B30" s="10"/>
       <c r="C30" s="10"/>
@@ -7257,7 +7164,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:33" x14ac:dyDescent="0.35">
       <c r="N32" s="55" t="s">
         <v>83</v>
       </c>
@@ -7266,7 +7173,7 @@
         <v>7224.33</v>
       </c>
     </row>
-    <row r="33" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B33" s="76"/>
       <c r="C33" s="76"/>
       <c r="D33" s="77"/>
@@ -7284,7 +7191,7 @@
         <v>7782.57</v>
       </c>
     </row>
-    <row r="34" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="34" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B34" s="78"/>
       <c r="C34" s="76"/>
       <c r="D34" s="77"/>
@@ -7503,20 +7410,20 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{240DD7AA-E2CC-4325-BB1A-65DAE33EC798}">
   <dimension ref="B2:R6"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="12.7109375" customWidth="1"/>
-    <col min="5" max="5" width="13.28515625" customWidth="1"/>
-    <col min="6" max="6" width="14.7109375" customWidth="1"/>
-    <col min="7" max="7" width="13.5703125" customWidth="1"/>
+    <col min="2" max="2" width="12.7265625" customWidth="1"/>
+    <col min="5" max="5" width="13.26953125" customWidth="1"/>
+    <col min="6" max="6" width="14.7265625" customWidth="1"/>
+    <col min="7" max="7" width="13.54296875" customWidth="1"/>
     <col min="8" max="15" width="0" hidden="1" customWidth="1"/>
-    <col min="16" max="16" width="16.140625" customWidth="1"/>
+    <col min="16" max="16" width="16.1796875" customWidth="1"/>
     <col min="17" max="17" width="0" hidden="1" customWidth="1"/>
     <col min="18" max="18" width="27" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="3" spans="2:18" ht="57" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:18" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
+    <row r="3" spans="2:18" ht="56" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B3" s="56" t="s">
         <v>52</v>
       </c>
@@ -7569,7 +7476,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="4" spans="2:18" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:18" ht="60" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B4" s="60" t="s">
         <v>68</v>
       </c>
@@ -7612,11 +7519,11 @@
       <c r="Q4" s="70">
         <v>0</v>
       </c>
-      <c r="R4" s="216" t="s">
+      <c r="R4" s="214" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="5" spans="2:18" ht="30" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:18" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B5" s="60" t="s">
         <v>68</v>
       </c>
@@ -7655,14 +7562,14 @@
       <c r="Q5" s="70">
         <v>0</v>
       </c>
-      <c r="R5" s="217"/>
-    </row>
-    <row r="6" spans="2:18" s="75" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B6" s="218" t="s">
+      <c r="R5" s="215"/>
+    </row>
+    <row r="6" spans="2:18" s="75" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="B6" s="216" t="s">
         <v>29</v>
       </c>
-      <c r="C6" s="219"/>
-      <c r="D6" s="220"/>
+      <c r="C6" s="217"/>
+      <c r="D6" s="218"/>
       <c r="E6" s="73">
         <v>160</v>
       </c>
@@ -7703,40 +7610,40 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AK50"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="4.5703125" style="4" customWidth="1"/>
-    <col min="2" max="2" width="11.85546875" style="1" customWidth="1"/>
-    <col min="3" max="3" width="11.28515625" style="1" customWidth="1"/>
-    <col min="4" max="4" width="12.5703125" style="4" customWidth="1"/>
-    <col min="5" max="5" width="20.7109375" style="4" customWidth="1"/>
-    <col min="6" max="6" width="12.7109375" style="4" customWidth="1"/>
-    <col min="7" max="7" width="18.42578125" style="4" customWidth="1"/>
-    <col min="8" max="8" width="19.42578125" style="4" customWidth="1"/>
-    <col min="9" max="9" width="12.7109375" style="4" customWidth="1"/>
-    <col min="10" max="10" width="11.85546875" style="4" customWidth="1"/>
-    <col min="11" max="11" width="14.7109375" style="4" customWidth="1"/>
-    <col min="12" max="12" width="16.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="10.7109375" style="1" customWidth="1"/>
-    <col min="14" max="14" width="13.140625" style="1" customWidth="1"/>
-    <col min="15" max="15" width="16.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="18.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="17" max="18" width="15.5703125" style="1" customWidth="1"/>
-    <col min="19" max="19" width="3.140625" style="1" customWidth="1"/>
-    <col min="20" max="20" width="28.140625" style="1" customWidth="1"/>
-    <col min="21" max="21" width="3.140625" style="1" customWidth="1"/>
-    <col min="22" max="27" width="8.7109375" style="1" customWidth="1"/>
-    <col min="28" max="28" width="3.140625" style="1" customWidth="1"/>
-    <col min="29" max="29" width="14.28515625" style="1" customWidth="1"/>
-    <col min="30" max="30" width="13.28515625" style="1" customWidth="1"/>
-    <col min="31" max="32" width="10.7109375" style="1" customWidth="1"/>
-    <col min="33" max="33" width="11.28515625" style="1" customWidth="1"/>
-    <col min="34" max="34" width="8.140625" style="1" customWidth="1"/>
-    <col min="35" max="35" width="38.140625" style="1" customWidth="1"/>
-    <col min="36" max="16384" width="9.140625" style="1"/>
+    <col min="1" max="1" width="4.54296875" style="4" customWidth="1"/>
+    <col min="2" max="2" width="11.81640625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="11.26953125" style="1" customWidth="1"/>
+    <col min="4" max="4" width="12.54296875" style="4" customWidth="1"/>
+    <col min="5" max="5" width="20.7265625" style="4" customWidth="1"/>
+    <col min="6" max="6" width="12.7265625" style="4" customWidth="1"/>
+    <col min="7" max="7" width="18.453125" style="4" customWidth="1"/>
+    <col min="8" max="8" width="19.453125" style="4" customWidth="1"/>
+    <col min="9" max="9" width="12.7265625" style="4" customWidth="1"/>
+    <col min="10" max="10" width="11.81640625" style="4" customWidth="1"/>
+    <col min="11" max="11" width="14.7265625" style="4" customWidth="1"/>
+    <col min="12" max="12" width="16.1796875" style="1" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="10.7265625" style="1" customWidth="1"/>
+    <col min="14" max="14" width="13.1796875" style="1" customWidth="1"/>
+    <col min="15" max="15" width="16.7265625" style="1" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="18.453125" style="1" bestFit="1" customWidth="1"/>
+    <col min="17" max="18" width="15.54296875" style="1" customWidth="1"/>
+    <col min="19" max="19" width="3.1796875" style="1" customWidth="1"/>
+    <col min="20" max="20" width="28.1796875" style="1" customWidth="1"/>
+    <col min="21" max="21" width="3.1796875" style="1" customWidth="1"/>
+    <col min="22" max="27" width="8.7265625" style="1" customWidth="1"/>
+    <col min="28" max="28" width="3.1796875" style="1" customWidth="1"/>
+    <col min="29" max="29" width="14.26953125" style="1" customWidth="1"/>
+    <col min="30" max="30" width="13.26953125" style="1" customWidth="1"/>
+    <col min="31" max="32" width="10.7265625" style="1" customWidth="1"/>
+    <col min="33" max="33" width="11.26953125" style="1" customWidth="1"/>
+    <col min="34" max="34" width="8.1796875" style="1" customWidth="1"/>
+    <col min="35" max="35" width="38.1796875" style="1" customWidth="1"/>
+    <col min="36" max="16384" width="9.1796875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:37" ht="45" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:37" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A1" s="126" t="s">
         <v>4</v>
       </c>
@@ -7786,7 +7693,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="2" spans="1:37" s="143" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:37" s="143" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A2" s="135">
         <v>1</v>
       </c>
@@ -7837,7 +7744,7 @@
       </c>
       <c r="P2" s="142"/>
     </row>
-    <row r="3" spans="1:37" s="143" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:37" s="143" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A3" s="135">
         <v>2</v>
       </c>
@@ -7906,7 +7813,7 @@
       <c r="AH3" s="144"/>
       <c r="AI3" s="146"/>
     </row>
-    <row r="4" spans="1:37" s="143" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:37" s="143" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A4" s="135">
         <v>3</v>
       </c>
@@ -7975,7 +7882,7 @@
       <c r="AH4" s="146"/>
       <c r="AI4" s="146"/>
     </row>
-    <row r="5" spans="1:37" s="143" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:37" s="143" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A5" s="135">
         <v>4</v>
       </c>
@@ -8042,7 +7949,7 @@
       <c r="AH5" s="155"/>
       <c r="AI5" s="156"/>
     </row>
-    <row r="6" spans="1:37" s="143" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:37" s="143" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A6" s="135">
         <v>5</v>
       </c>
@@ -8111,7 +8018,7 @@
       <c r="AH6" s="155"/>
       <c r="AI6" s="156"/>
     </row>
-    <row r="7" spans="1:37" s="143" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:37" s="143" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A7" s="135">
         <v>6</v>
       </c>
@@ -8178,7 +8085,7 @@
       <c r="AH7" s="155"/>
       <c r="AI7" s="156"/>
     </row>
-    <row r="8" spans="1:37" s="143" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:37" s="143" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A8" s="135">
         <v>7</v>
       </c>
@@ -8245,7 +8152,7 @@
       <c r="AH8" s="155"/>
       <c r="AI8" s="156"/>
     </row>
-    <row r="9" spans="1:37" s="143" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:37" s="143" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A9" s="135">
         <v>8</v>
       </c>
@@ -8312,7 +8219,7 @@
       <c r="AH9" s="155"/>
       <c r="AI9" s="156"/>
     </row>
-    <row r="10" spans="1:37" s="143" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:37" s="143" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A10" s="135">
         <v>9</v>
       </c>
@@ -8380,7 +8287,7 @@
       <c r="AI10" s="156"/>
       <c r="AK10" s="142"/>
     </row>
-    <row r="11" spans="1:37" s="143" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:37" s="143" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A11" s="135">
         <v>10</v>
       </c>
@@ -8447,7 +8354,7 @@
       <c r="AH11" s="155"/>
       <c r="AI11" s="156"/>
     </row>
-    <row r="12" spans="1:37" s="143" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:37" s="143" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A12" s="135">
         <v>11</v>
       </c>
@@ -8514,7 +8421,7 @@
       <c r="AH12" s="155"/>
       <c r="AI12" s="156"/>
     </row>
-    <row r="13" spans="1:37" s="143" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:37" s="143" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A13" s="135">
         <v>12</v>
       </c>
@@ -8581,7 +8488,7 @@
       <c r="AH13" s="155"/>
       <c r="AI13" s="156"/>
     </row>
-    <row r="14" spans="1:37" s="143" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:37" s="143" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A14" s="135">
         <v>13</v>
       </c>
@@ -8648,7 +8555,7 @@
       <c r="AH14" s="155"/>
       <c r="AI14" s="156"/>
     </row>
-    <row r="15" spans="1:37" s="143" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:37" s="143" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A15" s="135">
         <v>14</v>
       </c>
@@ -8717,7 +8624,7 @@
       <c r="AH15" s="155"/>
       <c r="AI15" s="156"/>
     </row>
-    <row r="16" spans="1:37" s="143" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:37" s="143" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A16" s="135">
         <v>15</v>
       </c>
@@ -8786,7 +8693,7 @@
       <c r="AH16" s="155"/>
       <c r="AI16" s="156"/>
     </row>
-    <row r="17" spans="1:35" s="143" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:35" s="143" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A17" s="135">
         <v>16</v>
       </c>
@@ -8855,7 +8762,7 @@
       <c r="AH17" s="155"/>
       <c r="AI17" s="156"/>
     </row>
-    <row r="18" spans="1:35" s="143" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:35" s="143" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A18" s="135">
         <v>17</v>
       </c>
@@ -8922,7 +8829,7 @@
       <c r="AH18" s="155"/>
       <c r="AI18" s="156"/>
     </row>
-    <row r="19" spans="1:35" s="143" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:35" s="143" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A19" s="135">
         <v>18</v>
       </c>
@@ -8989,7 +8896,7 @@
       <c r="AH19" s="155"/>
       <c r="AI19" s="156"/>
     </row>
-    <row r="20" spans="1:35" s="143" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:35" s="143" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A20" s="135">
         <v>19</v>
       </c>
@@ -9055,7 +8962,7 @@
       <c r="AH20" s="155"/>
       <c r="AI20" s="156"/>
     </row>
-    <row r="21" spans="1:35" s="143" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:35" s="143" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A21" s="135">
         <v>20</v>
       </c>
@@ -9122,7 +9029,7 @@
       <c r="AH21" s="155"/>
       <c r="AI21" s="156"/>
     </row>
-    <row r="22" spans="1:35" s="143" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:35" s="143" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A22" s="135">
         <v>21</v>
       </c>
@@ -9189,7 +9096,7 @@
       <c r="AH22" s="155"/>
       <c r="AI22" s="156"/>
     </row>
-    <row r="23" spans="1:35" s="143" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:35" s="143" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A23" s="135">
         <v>22</v>
       </c>
@@ -9256,7 +9163,7 @@
       <c r="AH23" s="155"/>
       <c r="AI23" s="156"/>
     </row>
-    <row r="24" spans="1:35" s="143" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:35" s="143" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A24" s="135">
         <v>23</v>
       </c>
@@ -9323,7 +9230,7 @@
       <c r="AH24" s="155"/>
       <c r="AI24" s="156"/>
     </row>
-    <row r="25" spans="1:35" s="143" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:35" s="143" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A25" s="135">
         <v>24</v>
       </c>
@@ -9390,7 +9297,7 @@
       <c r="AH25" s="155"/>
       <c r="AI25" s="156"/>
     </row>
-    <row r="26" spans="1:35" s="143" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:35" s="143" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A26" s="135">
         <v>25</v>
       </c>
@@ -9457,7 +9364,7 @@
       <c r="AH26" s="155"/>
       <c r="AI26" s="156"/>
     </row>
-    <row r="27" spans="1:35" s="143" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:35" s="143" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A27" s="135">
         <v>26</v>
       </c>
@@ -9524,7 +9431,7 @@
       <c r="AH27" s="155"/>
       <c r="AI27" s="156"/>
     </row>
-    <row r="28" spans="1:35" s="143" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:35" s="143" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A28" s="135">
         <v>27</v>
       </c>
@@ -9591,7 +9498,7 @@
       <c r="AH28" s="155"/>
       <c r="AI28" s="156"/>
     </row>
-    <row r="29" spans="1:35" s="143" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:35" s="143" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A29" s="135">
         <v>28</v>
       </c>
@@ -9658,7 +9565,7 @@
       <c r="AH29" s="155"/>
       <c r="AI29" s="156"/>
     </row>
-    <row r="30" spans="1:35" s="143" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:35" s="143" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A30" s="135">
         <v>29</v>
       </c>
@@ -9725,7 +9632,7 @@
       <c r="AH30" s="155"/>
       <c r="AI30" s="156"/>
     </row>
-    <row r="31" spans="1:35" s="143" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:35" s="143" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A31" s="135">
         <v>30</v>
       </c>
@@ -9792,7 +9699,7 @@
       <c r="AH31" s="155"/>
       <c r="AI31" s="156"/>
     </row>
-    <row r="32" spans="1:35" s="143" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:35" s="143" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A32" s="135">
         <v>31</v>
       </c>
@@ -9859,7 +9766,7 @@
       <c r="AH32" s="155"/>
       <c r="AI32" s="156"/>
     </row>
-    <row r="33" spans="1:35" s="143" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:35" s="143" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A33" s="135">
         <v>32</v>
       </c>
@@ -9927,7 +9834,7 @@
       <c r="AH33" s="155"/>
       <c r="AI33" s="156"/>
     </row>
-    <row r="34" spans="1:35" s="143" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:35" s="143" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A34" s="135">
         <v>33</v>
       </c>
@@ -9996,7 +9903,7 @@
       <c r="AH34" s="155"/>
       <c r="AI34" s="156"/>
     </row>
-    <row r="35" spans="1:35" s="143" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:35" s="143" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A35" s="135">
         <v>34</v>
       </c>
@@ -10065,7 +9972,7 @@
       <c r="AH35" s="155"/>
       <c r="AI35" s="156"/>
     </row>
-    <row r="36" spans="1:35" s="143" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:35" s="143" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A36" s="135">
         <v>35</v>
       </c>
@@ -10134,7 +10041,7 @@
       <c r="AH36" s="155"/>
       <c r="AI36" s="156"/>
     </row>
-    <row r="37" spans="1:35" s="143" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:35" s="143" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A37" s="135">
         <v>36</v>
       </c>
@@ -10202,7 +10109,7 @@
       <c r="AH37" s="155"/>
       <c r="AI37" s="156"/>
     </row>
-    <row r="38" spans="1:35" s="143" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:35" s="143" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A38" s="135">
         <v>37</v>
       </c>
@@ -10271,7 +10178,7 @@
       <c r="AH38" s="155"/>
       <c r="AI38" s="156"/>
     </row>
-    <row r="39" spans="1:35" s="143" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:35" s="143" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A39" s="135">
         <v>38</v>
       </c>
@@ -10340,7 +10247,7 @@
       <c r="AH39" s="155"/>
       <c r="AI39" s="156"/>
     </row>
-    <row r="40" spans="1:35" s="143" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:35" s="143" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A40" s="135">
         <v>39</v>
       </c>
@@ -10407,7 +10314,7 @@
       <c r="AH40" s="155"/>
       <c r="AI40" s="156"/>
     </row>
-    <row r="41" spans="1:35" s="143" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:35" s="143" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A41" s="135">
         <v>40</v>
       </c>
@@ -10474,7 +10381,7 @@
       <c r="AH41" s="155"/>
       <c r="AI41" s="156"/>
     </row>
-    <row r="42" spans="1:35" s="143" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:35" s="143" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A42" s="135">
         <v>41</v>
       </c>
@@ -10541,7 +10448,7 @@
       <c r="AH42" s="155"/>
       <c r="AI42" s="156"/>
     </row>
-    <row r="43" spans="1:35" s="143" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:35" s="143" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A43" s="135">
         <v>42</v>
       </c>
@@ -10608,7 +10515,7 @@
       <c r="AH43" s="155"/>
       <c r="AI43" s="156"/>
     </row>
-    <row r="44" spans="1:35" s="143" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:35" s="143" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A44" s="135">
         <v>43</v>
       </c>
@@ -10675,7 +10582,7 @@
       <c r="AH44" s="155"/>
       <c r="AI44" s="156"/>
     </row>
-    <row r="45" spans="1:35" s="143" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:35" s="143" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A45" s="135">
         <v>44</v>
       </c>
@@ -10743,7 +10650,7 @@
       <c r="AH45" s="155"/>
       <c r="AI45" s="156"/>
     </row>
-    <row r="46" spans="1:35" s="143" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:35" s="143" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A46" s="135">
         <v>45</v>
       </c>
@@ -10812,7 +10719,7 @@
       <c r="AH46" s="155"/>
       <c r="AI46" s="156"/>
     </row>
-    <row r="47" spans="1:35" s="143" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:35" s="143" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A47" s="135">
         <v>46</v>
       </c>
@@ -10881,7 +10788,7 @@
       <c r="AH47" s="155"/>
       <c r="AI47" s="156"/>
     </row>
-    <row r="48" spans="1:35" s="143" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:35" s="143" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A48" s="135">
         <v>47</v>
       </c>
@@ -10949,7 +10856,7 @@
       <c r="AH48" s="148"/>
       <c r="AI48" s="148"/>
     </row>
-    <row r="49" spans="1:35" s="143" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:35" s="143" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A49" s="135">
         <v>48</v>
       </c>
@@ -11018,7 +10925,7 @@
       <c r="AH49" s="155"/>
       <c r="AI49" s="156"/>
     </row>
-    <row r="50" spans="1:35" s="143" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:35" s="143" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A50" s="135">
         <v>49</v>
       </c>
@@ -11165,375 +11072,454 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3E3F0E1F-80A5-4555-9FE1-744B1DEBC4EC}">
-  <dimension ref="B1:L15"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="B1:P15"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="1.28515625" customWidth="1"/>
-    <col min="3" max="3" width="20.85546875" customWidth="1"/>
-    <col min="4" max="4" width="13.42578125" customWidth="1"/>
-    <col min="5" max="5" width="14.5703125" customWidth="1"/>
-    <col min="6" max="6" width="11.140625" customWidth="1"/>
-    <col min="7" max="7" width="13.42578125" customWidth="1"/>
-    <col min="8" max="8" width="12.5703125" customWidth="1"/>
-    <col min="9" max="9" width="15.140625" customWidth="1"/>
-    <col min="10" max="10" width="11.140625" customWidth="1"/>
+    <col min="1" max="1" width="1.26953125" customWidth="1"/>
+    <col min="3" max="3" width="20.81640625" customWidth="1"/>
+    <col min="4" max="4" width="13.453125" customWidth="1"/>
+    <col min="5" max="5" width="14.54296875" customWidth="1"/>
+    <col min="6" max="6" width="11.1796875" customWidth="1"/>
+    <col min="7" max="7" width="13.453125" customWidth="1"/>
+    <col min="8" max="8" width="12.54296875" customWidth="1"/>
+    <col min="9" max="9" width="15.1796875" customWidth="1"/>
+    <col min="10" max="10" width="11.1796875" customWidth="1"/>
     <col min="11" max="11" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B1" s="221" t="s">
+    <row r="1" spans="2:16" x14ac:dyDescent="0.35">
+      <c r="B1" s="219" t="s">
         <v>198</v>
       </c>
-      <c r="C1" s="221"/>
-      <c r="D1" s="221"/>
-      <c r="E1" s="221"/>
-      <c r="F1" s="221"/>
-      <c r="G1" s="221"/>
-      <c r="H1" s="221"/>
-      <c r="I1" s="221"/>
-      <c r="J1" s="221"/>
-      <c r="K1" s="221"/>
-      <c r="L1" s="221"/>
-    </row>
-    <row r="2" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B2" s="222" t="s">
+      <c r="C1" s="219"/>
+      <c r="D1" s="219"/>
+      <c r="E1" s="219"/>
+      <c r="F1" s="219"/>
+      <c r="G1" s="219"/>
+      <c r="H1" s="219"/>
+      <c r="I1" s="219"/>
+      <c r="J1" s="219"/>
+      <c r="K1" s="219"/>
+      <c r="L1" s="219"/>
+    </row>
+    <row r="2" spans="2:16" x14ac:dyDescent="0.35">
+      <c r="B2" s="220" t="s">
         <v>199</v>
       </c>
-      <c r="C2" s="222"/>
-      <c r="D2" s="222"/>
-      <c r="E2" s="222"/>
-      <c r="F2" s="222"/>
-      <c r="G2" s="222"/>
-      <c r="H2" s="222"/>
-      <c r="I2" s="222"/>
-      <c r="J2" s="222"/>
-      <c r="K2" s="222"/>
-      <c r="L2" s="222"/>
-    </row>
-    <row r="3" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B3" s="223" t="s">
+      <c r="C2" s="220"/>
+      <c r="D2" s="220"/>
+      <c r="E2" s="220"/>
+      <c r="F2" s="220"/>
+      <c r="G2" s="220"/>
+      <c r="H2" s="220"/>
+      <c r="I2" s="220"/>
+      <c r="J2" s="220"/>
+      <c r="K2" s="220"/>
+      <c r="L2" s="220"/>
+    </row>
+    <row r="3" spans="2:16" x14ac:dyDescent="0.35">
+      <c r="B3" s="221" t="s">
         <v>200</v>
       </c>
-      <c r="C3" s="223"/>
-      <c r="D3" s="223"/>
-      <c r="E3" s="223"/>
-      <c r="F3" s="223"/>
-      <c r="G3" s="223"/>
-      <c r="H3" s="223"/>
-      <c r="I3" s="223"/>
-      <c r="J3" s="223"/>
-      <c r="K3" s="223"/>
-      <c r="L3" s="223"/>
-    </row>
-    <row r="4" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="224" t="s">
+      <c r="C3" s="221"/>
+      <c r="D3" s="221"/>
+      <c r="E3" s="221"/>
+      <c r="F3" s="221"/>
+      <c r="G3" s="221"/>
+      <c r="H3" s="221"/>
+      <c r="I3" s="221"/>
+      <c r="J3" s="221"/>
+      <c r="K3" s="221"/>
+      <c r="L3" s="221"/>
+    </row>
+    <row r="4" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B4" s="222" t="s">
         <v>201</v>
       </c>
-      <c r="C4" s="224"/>
-      <c r="D4" s="224"/>
-      <c r="E4" s="224"/>
-      <c r="F4" s="224"/>
-      <c r="G4" s="224"/>
-      <c r="H4" s="224"/>
-      <c r="I4" s="224"/>
-      <c r="J4" s="224"/>
-      <c r="K4" s="224"/>
-      <c r="L4" s="224"/>
-    </row>
-    <row r="5" spans="2:12" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B5" s="192" t="s">
+      <c r="C4" s="222"/>
+      <c r="D4" s="222"/>
+      <c r="E4" s="222"/>
+      <c r="F4" s="222"/>
+      <c r="G4" s="222"/>
+      <c r="H4" s="222"/>
+      <c r="I4" s="222"/>
+      <c r="J4" s="222"/>
+      <c r="K4" s="222"/>
+      <c r="L4" s="222"/>
+    </row>
+    <row r="5" spans="2:16" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B5" s="186" t="s">
+        <v>207</v>
+      </c>
+      <c r="C5" s="187"/>
+      <c r="D5" s="187"/>
+      <c r="E5" s="187"/>
+      <c r="F5" s="187"/>
+      <c r="G5" s="187"/>
+      <c r="H5" s="187"/>
+      <c r="I5" s="187"/>
+      <c r="J5" s="187"/>
+      <c r="K5" s="188"/>
+    </row>
+    <row r="6" spans="2:16" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="B6" s="190" t="s">
+        <v>208</v>
+      </c>
+      <c r="C6" s="190" t="s">
+        <v>209</v>
+      </c>
+      <c r="D6" s="190" t="s">
+        <v>210</v>
+      </c>
+      <c r="E6" s="190" t="s">
+        <v>211</v>
+      </c>
+      <c r="F6" s="190" t="s">
+        <v>212</v>
+      </c>
+      <c r="G6" s="190" t="s">
+        <v>213</v>
+      </c>
+      <c r="H6" s="190" t="s">
+        <v>202</v>
+      </c>
+      <c r="I6" s="190" t="s">
+        <v>203</v>
+      </c>
+      <c r="J6" s="190" t="s">
+        <v>204</v>
+      </c>
+      <c r="K6" s="190" t="s">
+        <v>214</v>
+      </c>
+      <c r="L6" s="190" t="s">
+        <v>215</v>
+      </c>
+      <c r="M6" s="190" t="s">
+        <v>112</v>
+      </c>
+      <c r="N6" s="190" t="s">
+        <v>216</v>
+      </c>
+      <c r="O6" s="190" t="s">
+        <v>109</v>
+      </c>
+      <c r="P6" s="190" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="7" spans="2:16" ht="29" x14ac:dyDescent="0.35">
+      <c r="B7" s="191">
+        <v>1</v>
+      </c>
+      <c r="C7" s="191">
+        <v>6</v>
+      </c>
+      <c r="D7" s="227" t="s">
+        <v>230</v>
+      </c>
+      <c r="E7" s="191">
+        <v>4901.2359999999999</v>
+      </c>
+      <c r="F7" s="191" t="s">
+        <v>217</v>
+      </c>
+      <c r="G7" s="191">
+        <v>13</v>
+      </c>
+      <c r="H7" s="192">
+        <v>45967</v>
+      </c>
+      <c r="I7" s="192">
+        <v>45968</v>
+      </c>
+      <c r="J7" s="192">
+        <v>45972</v>
+      </c>
+      <c r="K7" s="192">
+        <v>45974</v>
+      </c>
+      <c r="L7" s="191" t="s">
+        <v>218</v>
+      </c>
+      <c r="M7" s="191" t="s">
+        <v>205</v>
+      </c>
+      <c r="N7" s="191"/>
+      <c r="O7" s="191" t="s">
         <v>220</v>
       </c>
-      <c r="C5" s="193"/>
-      <c r="D5" s="193"/>
-      <c r="E5" s="193"/>
-      <c r="F5" s="193"/>
-      <c r="G5" s="193"/>
-      <c r="H5" s="193"/>
-      <c r="I5" s="193"/>
-      <c r="J5" s="193"/>
-      <c r="K5" s="194"/>
-    </row>
-    <row r="6" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B6" s="233" t="s">
-        <v>202</v>
-      </c>
-      <c r="C6" s="225" t="s">
-        <v>203</v>
-      </c>
-      <c r="D6" s="225" t="s">
+      <c r="P7" s="191" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="8" spans="2:16" ht="29" x14ac:dyDescent="0.35">
+      <c r="B8" s="191">
+        <v>2</v>
+      </c>
+      <c r="C8" s="191">
+        <v>5</v>
+      </c>
+      <c r="D8" s="191" t="s">
+        <v>225</v>
+      </c>
+      <c r="E8" s="191">
+        <v>4418.3890000000001</v>
+      </c>
+      <c r="F8" s="191" t="s">
+        <v>217</v>
+      </c>
+      <c r="G8" s="191">
+        <v>11</v>
+      </c>
+      <c r="H8" s="192">
+        <v>45977</v>
+      </c>
+      <c r="I8" s="192">
+        <v>45978</v>
+      </c>
+      <c r="J8" s="192">
+        <v>45981</v>
+      </c>
+      <c r="K8" s="192">
+        <v>45983</v>
+      </c>
+      <c r="L8" s="191" t="s">
+        <v>218</v>
+      </c>
+      <c r="M8" s="191" t="s">
+        <v>205</v>
+      </c>
+      <c r="N8" s="191"/>
+      <c r="O8" s="191" t="s">
+        <v>220</v>
+      </c>
+      <c r="P8" s="191" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="9" spans="2:16" ht="29" x14ac:dyDescent="0.35">
+      <c r="B9" s="191">
+        <v>3</v>
+      </c>
+      <c r="C9" s="191" t="s">
+        <v>225</v>
+      </c>
+      <c r="D9" s="191">
+        <v>6</v>
+      </c>
+      <c r="E9" s="191">
+        <v>419.48</v>
+      </c>
+      <c r="F9" s="191" t="s">
+        <v>217</v>
+      </c>
+      <c r="G9" s="191">
+        <v>1</v>
+      </c>
+      <c r="H9" s="192">
+        <v>45984</v>
+      </c>
+      <c r="I9" s="192">
+        <v>45985</v>
+      </c>
+      <c r="J9" s="192">
+        <v>45988</v>
+      </c>
+      <c r="K9" s="192">
+        <v>45990</v>
+      </c>
+      <c r="L9" s="191" t="s">
+        <v>218</v>
+      </c>
+      <c r="M9" s="191" t="s">
+        <v>205</v>
+      </c>
+      <c r="N9" s="191"/>
+      <c r="O9" s="191" t="s">
         <v>221</v>
       </c>
-      <c r="E6" s="225" t="s">
-        <v>204</v>
-      </c>
-      <c r="F6" s="225" t="s">
-        <v>205</v>
-      </c>
-      <c r="G6" s="225" t="s">
+      <c r="P9" s="191" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="10" spans="2:16" ht="29" x14ac:dyDescent="0.35">
+      <c r="B10" s="191">
+        <v>4</v>
+      </c>
+      <c r="C10" s="191" t="s">
+        <v>226</v>
+      </c>
+      <c r="D10" s="191" t="s">
+        <v>227</v>
+      </c>
+      <c r="E10" s="191">
+        <v>840.43899999999996</v>
+      </c>
+      <c r="F10" s="191" t="s">
+        <v>217</v>
+      </c>
+      <c r="G10" s="191">
+        <v>2</v>
+      </c>
+      <c r="H10" s="192">
+        <v>45971</v>
+      </c>
+      <c r="I10" s="192">
+        <v>45973</v>
+      </c>
+      <c r="J10" s="192">
+        <v>45976</v>
+      </c>
+      <c r="K10" s="192">
+        <v>45979</v>
+      </c>
+      <c r="L10" s="191" t="s">
+        <v>219</v>
+      </c>
+      <c r="M10" s="191" t="s">
         <v>206</v>
       </c>
-      <c r="H6" s="225" t="s">
-        <v>207</v>
-      </c>
-      <c r="I6" s="225" t="s">
-        <v>208</v>
-      </c>
-      <c r="J6" s="225" t="s">
-        <v>209</v>
-      </c>
-      <c r="K6" s="235" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="7" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B7" s="234"/>
-      <c r="C7" s="226"/>
-      <c r="D7" s="226"/>
-      <c r="E7" s="226"/>
-      <c r="F7" s="226"/>
-      <c r="G7" s="226"/>
-      <c r="H7" s="226"/>
-      <c r="I7" s="226"/>
-      <c r="J7" s="226"/>
-      <c r="K7" s="236"/>
-    </row>
-    <row r="8" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B8" s="189">
-        <v>1</v>
-      </c>
-      <c r="C8" s="190" t="s">
-        <v>210</v>
-      </c>
-      <c r="D8" s="191">
-        <v>4901.2360000000008</v>
-      </c>
-      <c r="E8" s="191" t="s">
-        <v>211</v>
-      </c>
-      <c r="F8" s="191">
-        <v>13</v>
-      </c>
-      <c r="G8" s="133">
-        <v>45967</v>
-      </c>
-      <c r="H8" s="133">
-        <v>45968</v>
-      </c>
-      <c r="I8" s="133">
-        <v>45972</v>
-      </c>
-      <c r="J8" s="133">
-        <v>45974</v>
-      </c>
-      <c r="K8" s="227" t="s">
-        <v>212</v>
-      </c>
-      <c r="L8" s="173"/>
-    </row>
-    <row r="9" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B9" s="181">
-        <v>2</v>
-      </c>
-      <c r="C9" s="182" t="s">
-        <v>213</v>
-      </c>
-      <c r="D9" s="135">
-        <v>4418.3890000000001</v>
-      </c>
-      <c r="E9" s="135" t="s">
-        <v>211</v>
-      </c>
-      <c r="F9" s="135">
-        <v>11</v>
-      </c>
-      <c r="G9" s="133">
-        <v>45977</v>
-      </c>
-      <c r="H9" s="133">
-        <v>45978</v>
-      </c>
-      <c r="I9" s="133">
-        <v>45981</v>
-      </c>
-      <c r="J9" s="133">
+      <c r="N10" s="191"/>
+      <c r="O10" s="191" t="s">
+        <v>221</v>
+      </c>
+      <c r="P10" s="191" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="11" spans="2:16" ht="29" x14ac:dyDescent="0.35">
+      <c r="B11" s="191">
+        <v>5</v>
+      </c>
+      <c r="C11" s="191" t="s">
+        <v>228</v>
+      </c>
+      <c r="D11" s="191" t="s">
+        <v>226</v>
+      </c>
+      <c r="E11" s="191">
+        <v>3283.51</v>
+      </c>
+      <c r="F11" s="191" t="s">
+        <v>217</v>
+      </c>
+      <c r="G11" s="191">
+        <v>8</v>
+      </c>
+      <c r="H11" s="192">
         <v>45983</v>
       </c>
-      <c r="K9" s="228"/>
-      <c r="L9" s="173"/>
-    </row>
-    <row r="10" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B10" s="181">
-        <v>3</v>
-      </c>
-      <c r="C10" s="182" t="s">
-        <v>214</v>
-      </c>
-      <c r="D10" s="135">
-        <v>419.48</v>
-      </c>
-      <c r="E10" s="135" t="s">
-        <v>211</v>
-      </c>
-      <c r="F10" s="135">
-        <v>1</v>
-      </c>
-      <c r="G10" s="133">
+      <c r="I11" s="192">
         <v>45984</v>
       </c>
-      <c r="H10" s="133">
-        <v>45985</v>
-      </c>
-      <c r="I10" s="133">
+      <c r="J11" s="192">
+        <v>45987</v>
+      </c>
+      <c r="K11" s="192">
+        <v>45989</v>
+      </c>
+      <c r="L11" s="191" t="s">
+        <v>219</v>
+      </c>
+      <c r="M11" s="191" t="s">
+        <v>206</v>
+      </c>
+      <c r="N11" s="191"/>
+      <c r="O11" s="191" t="s">
+        <v>222</v>
+      </c>
+      <c r="P11" s="191" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="12" spans="2:16" ht="29" x14ac:dyDescent="0.35">
+      <c r="B12" s="191">
+        <v>6</v>
+      </c>
+      <c r="C12" s="191" t="s">
+        <v>227</v>
+      </c>
+      <c r="D12" s="191" t="s">
+        <v>229</v>
+      </c>
+      <c r="E12" s="191">
+        <v>4049.7640000000001</v>
+      </c>
+      <c r="F12" s="191" t="s">
+        <v>217</v>
+      </c>
+      <c r="G12" s="191">
+        <v>10</v>
+      </c>
+      <c r="H12" s="192">
         <v>45988</v>
       </c>
-      <c r="J10" s="133">
-        <v>45990</v>
-      </c>
-      <c r="K10" s="229"/>
-      <c r="L10" s="173"/>
-    </row>
-    <row r="11" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B11" s="180">
-        <v>4</v>
-      </c>
-      <c r="C11" s="174" t="s">
-        <v>215</v>
-      </c>
-      <c r="D11" s="8">
-        <v>840.43900000000008</v>
-      </c>
-      <c r="E11" s="183" t="s">
-        <v>211</v>
-      </c>
-      <c r="F11" s="8">
-        <v>2</v>
-      </c>
-      <c r="G11" s="133">
-        <v>45971</v>
-      </c>
-      <c r="H11" s="133">
-        <v>45973</v>
-      </c>
-      <c r="I11" s="133">
-        <v>45976</v>
-      </c>
-      <c r="J11" s="133">
-        <v>45979</v>
-      </c>
-      <c r="K11" s="230" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="12" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B12" s="180">
-        <v>5</v>
-      </c>
-      <c r="C12" s="174" t="s">
-        <v>217</v>
-      </c>
-      <c r="D12" s="8">
-        <v>3283.51</v>
-      </c>
-      <c r="E12" s="183" t="s">
-        <v>211</v>
-      </c>
-      <c r="F12" s="8">
-        <v>8</v>
-      </c>
-      <c r="G12" s="133">
-        <v>45983</v>
-      </c>
-      <c r="H12" s="133">
-        <v>45984</v>
-      </c>
-      <c r="I12" s="133">
-        <v>45987</v>
-      </c>
-      <c r="J12" s="133">
+      <c r="I12" s="192">
         <v>45989</v>
       </c>
-      <c r="K12" s="231"/>
-    </row>
-    <row r="13" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B13" s="180">
-        <v>6</v>
-      </c>
-      <c r="C13" s="174" t="s">
-        <v>218</v>
-      </c>
-      <c r="D13" s="8">
-        <v>4049.7639999999997</v>
-      </c>
-      <c r="E13" s="183" t="s">
-        <v>211</v>
-      </c>
-      <c r="F13" s="8">
-        <v>10</v>
-      </c>
-      <c r="G13" s="133">
-        <v>45988</v>
-      </c>
-      <c r="H13" s="133">
-        <f>G13+1</f>
-        <v>45989</v>
-      </c>
-      <c r="I13" s="133">
+      <c r="J12" s="192">
         <v>45991</v>
       </c>
-      <c r="J13" s="133">
+      <c r="K12" s="192">
         <v>45995</v>
       </c>
-      <c r="K13" s="232"/>
-    </row>
-    <row r="14" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B14" s="185"/>
-      <c r="C14" s="186"/>
-      <c r="D14" s="186"/>
-      <c r="E14" s="187"/>
+      <c r="L12" s="191" t="s">
+        <v>219</v>
+      </c>
+      <c r="M12" s="191" t="s">
+        <v>206</v>
+      </c>
+      <c r="N12" s="191"/>
+      <c r="O12" s="191" t="s">
+        <v>222</v>
+      </c>
+      <c r="P12" s="191" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="13" spans="2:16" x14ac:dyDescent="0.35">
+      <c r="B13" s="179"/>
+      <c r="C13" s="173"/>
+      <c r="D13" s="8"/>
+      <c r="E13" s="180"/>
+      <c r="F13" s="8"/>
+      <c r="G13" s="133"/>
+      <c r="H13" s="133"/>
+      <c r="I13" s="133"/>
+      <c r="J13" s="133"/>
+      <c r="K13" s="189"/>
+    </row>
+    <row r="14" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B14" s="182"/>
+      <c r="C14" s="183"/>
+      <c r="D14" s="183"/>
+      <c r="E14" s="184"/>
       <c r="F14" s="92"/>
       <c r="G14" s="92"/>
       <c r="H14" s="92"/>
       <c r="I14" s="92"/>
       <c r="J14" s="92"/>
-      <c r="K14" s="188"/>
-    </row>
-    <row r="15" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B15" s="176" t="s">
-        <v>219</v>
-      </c>
-      <c r="C15" s="177"/>
-      <c r="D15" s="184">
-        <v>17.912817999999998</v>
-      </c>
-      <c r="E15" s="178"/>
-      <c r="F15" s="179">
-        <v>45</v>
-      </c>
-      <c r="G15" s="179"/>
-      <c r="H15" s="179"/>
-      <c r="I15" s="179"/>
-      <c r="J15" s="179"/>
-      <c r="K15" s="175"/>
+      <c r="K14" s="185"/>
+    </row>
+    <row r="15" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B15" s="175"/>
+      <c r="C15" s="176"/>
+      <c r="D15" s="181"/>
+      <c r="E15" s="177"/>
+      <c r="F15" s="178"/>
+      <c r="G15" s="178"/>
+      <c r="H15" s="178"/>
+      <c r="I15" s="178"/>
+      <c r="J15" s="178"/>
+      <c r="K15" s="174"/>
     </row>
   </sheetData>
-  <mergeCells count="16">
-    <mergeCell ref="K8:K10"/>
-    <mergeCell ref="K11:K13"/>
-    <mergeCell ref="F6:F7"/>
-    <mergeCell ref="B6:B7"/>
-    <mergeCell ref="C6:C7"/>
-    <mergeCell ref="D6:D7"/>
-    <mergeCell ref="E6:E7"/>
-    <mergeCell ref="K6:K7"/>
+  <mergeCells count="4">
     <mergeCell ref="B1:L1"/>
     <mergeCell ref="B2:L2"/>
     <mergeCell ref="B3:L3"/>
     <mergeCell ref="B4:L4"/>
-    <mergeCell ref="G6:G7"/>
-    <mergeCell ref="H6:H7"/>
-    <mergeCell ref="I6:I7"/>
-    <mergeCell ref="J6:J7"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -11545,50 +11531,50 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB34"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="3.42578125" style="4" customWidth="1"/>
-    <col min="2" max="2" width="15.28515625" style="1" customWidth="1"/>
-    <col min="3" max="3" width="11.28515625" style="1" customWidth="1"/>
-    <col min="4" max="4" width="12.5703125" style="4" customWidth="1"/>
-    <col min="5" max="5" width="12.7109375" style="4" customWidth="1"/>
-    <col min="6" max="6" width="10.140625" style="4" customWidth="1"/>
-    <col min="7" max="7" width="12.5703125" style="4" customWidth="1"/>
-    <col min="8" max="8" width="11.5703125" style="1" customWidth="1"/>
-    <col min="9" max="10" width="10.7109375" style="1" customWidth="1"/>
-    <col min="11" max="11" width="14.85546875" style="1" customWidth="1"/>
-    <col min="12" max="12" width="3.140625" style="1" customWidth="1"/>
-    <col min="13" max="13" width="14.5703125" style="1" customWidth="1"/>
-    <col min="14" max="14" width="3.140625" style="1" customWidth="1"/>
-    <col min="15" max="15" width="10.5703125" style="1" customWidth="1"/>
-    <col min="16" max="20" width="8.7109375" style="1" customWidth="1"/>
-    <col min="21" max="21" width="3.140625" style="1" customWidth="1"/>
-    <col min="22" max="22" width="10.7109375" style="1" customWidth="1"/>
-    <col min="23" max="23" width="12.5703125" style="1" customWidth="1"/>
-    <col min="24" max="24" width="12.42578125" style="1" customWidth="1"/>
-    <col min="25" max="26" width="10.7109375" style="1" customWidth="1"/>
-    <col min="27" max="27" width="14.42578125" style="1" customWidth="1"/>
-    <col min="28" max="28" width="17.28515625" style="1" customWidth="1"/>
-    <col min="29" max="16384" width="9.140625" style="1"/>
+    <col min="1" max="1" width="3.453125" style="4" customWidth="1"/>
+    <col min="2" max="2" width="15.26953125" style="1" customWidth="1"/>
+    <col min="3" max="3" width="11.26953125" style="1" customWidth="1"/>
+    <col min="4" max="4" width="12.54296875" style="4" customWidth="1"/>
+    <col min="5" max="5" width="12.7265625" style="4" customWidth="1"/>
+    <col min="6" max="6" width="10.1796875" style="4" customWidth="1"/>
+    <col min="7" max="7" width="12.54296875" style="4" customWidth="1"/>
+    <col min="8" max="8" width="11.54296875" style="1" customWidth="1"/>
+    <col min="9" max="10" width="10.7265625" style="1" customWidth="1"/>
+    <col min="11" max="11" width="14.81640625" style="1" customWidth="1"/>
+    <col min="12" max="12" width="3.1796875" style="1" customWidth="1"/>
+    <col min="13" max="13" width="14.54296875" style="1" customWidth="1"/>
+    <col min="14" max="14" width="3.1796875" style="1" customWidth="1"/>
+    <col min="15" max="15" width="10.54296875" style="1" customWidth="1"/>
+    <col min="16" max="20" width="8.7265625" style="1" customWidth="1"/>
+    <col min="21" max="21" width="3.1796875" style="1" customWidth="1"/>
+    <col min="22" max="22" width="10.7265625" style="1" customWidth="1"/>
+    <col min="23" max="23" width="12.54296875" style="1" customWidth="1"/>
+    <col min="24" max="24" width="12.453125" style="1" customWidth="1"/>
+    <col min="25" max="26" width="10.7265625" style="1" customWidth="1"/>
+    <col min="27" max="27" width="14.453125" style="1" customWidth="1"/>
+    <col min="28" max="28" width="17.26953125" style="1" customWidth="1"/>
+    <col min="29" max="16384" width="9.1796875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A1" s="13" t="s">
         <v>0</v>
       </c>
       <c r="D1" s="38"/>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A2" s="13" t="s">
         <v>21</v>
       </c>
       <c r="D2" s="1"/>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A3" s="6"/>
       <c r="D3" s="1"/>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A4" s="13" t="s">
         <v>22</v>
       </c>
@@ -11605,7 +11591,7 @@
         <v>905812</v>
       </c>
     </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A5" s="6"/>
       <c r="D5" s="2" t="s">
         <v>29</v>
@@ -11615,7 +11601,7 @@
       </c>
       <c r="O5" s="118"/>
     </row>
-    <row r="6" spans="1:15" ht="17.25" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:15" ht="16" x14ac:dyDescent="0.35">
       <c r="A6" s="6"/>
       <c r="D6" s="2" t="s">
         <v>92</v>
@@ -11624,7 +11610,7 @@
         <v>32.6</v>
       </c>
     </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A7" s="6"/>
       <c r="D7" s="2" t="s">
         <v>2</v>
@@ -11634,11 +11620,11 @@
         <v>82.4</v>
       </c>
     </row>
-    <row r="8" spans="1:15" ht="5.0999999999999996" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:15" ht="5.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A8" s="6"/>
       <c r="D8" s="1"/>
     </row>
-    <row r="9" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A9" s="13" t="s">
         <v>23</v>
       </c>
@@ -11660,13 +11646,13 @@
         <v>32</v>
       </c>
     </row>
-    <row r="10" spans="1:15" ht="5.0999999999999996" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:15" ht="5.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="13"/>
       <c r="D10" s="1"/>
       <c r="E10" s="1"/>
       <c r="F10" s="13"/>
     </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A11" s="13" t="s">
         <v>33</v>
       </c>
@@ -11690,7 +11676,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A12" s="5"/>
       <c r="D12" s="2" t="s">
         <v>25</v>
@@ -11712,7 +11698,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A13" s="5"/>
       <c r="D13" s="2" t="s">
         <v>26</v>
@@ -11734,7 +11720,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A14" s="5"/>
       <c r="D14" s="2" t="s">
         <v>27</v>
@@ -11756,7 +11742,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:15" ht="17.25" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:15" ht="16" x14ac:dyDescent="0.35">
       <c r="A15" s="5"/>
       <c r="D15" s="28" t="s">
         <v>28</v>
@@ -11778,7 +11764,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A16" s="5"/>
       <c r="D16" s="27" t="s">
         <v>29</v>
@@ -11800,125 +11786,125 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A17" s="5"/>
       <c r="D17" s="6"/>
       <c r="E17" s="6"/>
       <c r="F17" s="6"/>
     </row>
-    <row r="18" spans="1:28" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="213" t="s">
+    <row r="18" spans="1:28" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A18" s="211" t="s">
         <v>4</v>
       </c>
-      <c r="B18" s="213" t="s">
+      <c r="B18" s="211" t="s">
         <v>42</v>
       </c>
-      <c r="C18" s="209" t="s">
+      <c r="C18" s="207" t="s">
         <v>47</v>
       </c>
-      <c r="D18" s="209" t="s">
+      <c r="D18" s="207" t="s">
         <v>43</v>
       </c>
-      <c r="E18" s="213" t="s">
+      <c r="E18" s="211" t="s">
         <v>8</v>
       </c>
-      <c r="F18" s="200" t="s">
+      <c r="F18" s="198" t="s">
         <v>18</v>
       </c>
-      <c r="G18" s="200"/>
-      <c r="H18" s="200"/>
-      <c r="I18" s="200"/>
-      <c r="J18" s="200"/>
-      <c r="K18" s="203" t="s">
+      <c r="G18" s="198"/>
+      <c r="H18" s="198"/>
+      <c r="I18" s="198"/>
+      <c r="J18" s="198"/>
+      <c r="K18" s="201" t="s">
         <v>19</v>
       </c>
-      <c r="M18" s="209" t="s">
+      <c r="M18" s="207" t="s">
         <v>36</v>
       </c>
-      <c r="O18" s="204" t="s">
+      <c r="O18" s="202" t="s">
         <v>31</v>
       </c>
-      <c r="P18" s="205"/>
-      <c r="Q18" s="205"/>
-      <c r="R18" s="205"/>
-      <c r="S18" s="205"/>
-      <c r="T18" s="206"/>
-      <c r="V18" s="204" t="s">
+      <c r="P18" s="203"/>
+      <c r="Q18" s="203"/>
+      <c r="R18" s="203"/>
+      <c r="S18" s="203"/>
+      <c r="T18" s="204"/>
+      <c r="V18" s="202" t="s">
         <v>30</v>
       </c>
-      <c r="W18" s="205"/>
-      <c r="X18" s="205"/>
-      <c r="Y18" s="205"/>
-      <c r="Z18" s="205"/>
-      <c r="AA18" s="206"/>
-      <c r="AB18" s="207" t="s">
+      <c r="W18" s="203"/>
+      <c r="X18" s="203"/>
+      <c r="Y18" s="203"/>
+      <c r="Z18" s="203"/>
+      <c r="AA18" s="204"/>
+      <c r="AB18" s="205" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="19" spans="1:28" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="214"/>
-      <c r="B19" s="214"/>
-      <c r="C19" s="211"/>
-      <c r="D19" s="214"/>
-      <c r="E19" s="214"/>
-      <c r="F19" s="237" t="s">
+    <row r="19" spans="1:28" ht="21" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A19" s="212"/>
+      <c r="B19" s="212"/>
+      <c r="C19" s="209"/>
+      <c r="D19" s="212"/>
+      <c r="E19" s="212"/>
+      <c r="F19" s="223" t="s">
         <v>40</v>
       </c>
-      <c r="G19" s="238" t="s">
+      <c r="G19" s="224" t="s">
         <v>44</v>
       </c>
-      <c r="H19" s="239"/>
-      <c r="I19" s="238" t="s">
+      <c r="H19" s="225"/>
+      <c r="I19" s="224" t="s">
         <v>45</v>
       </c>
-      <c r="J19" s="239"/>
-      <c r="K19" s="203"/>
-      <c r="M19" s="210"/>
-      <c r="O19" s="201" t="s">
+      <c r="J19" s="225"/>
+      <c r="K19" s="201"/>
+      <c r="M19" s="208"/>
+      <c r="O19" s="199" t="s">
         <v>24</v>
       </c>
-      <c r="P19" s="201" t="s">
+      <c r="P19" s="199" t="s">
         <v>25</v>
       </c>
-      <c r="Q19" s="201" t="s">
+      <c r="Q19" s="199" t="s">
         <v>26</v>
       </c>
-      <c r="R19" s="201" t="s">
+      <c r="R19" s="199" t="s">
         <v>27</v>
       </c>
-      <c r="S19" s="201" t="s">
+      <c r="S19" s="199" t="s">
         <v>28</v>
       </c>
       <c r="T19" s="43" t="s">
         <v>29</v>
       </c>
-      <c r="V19" s="201" t="s">
+      <c r="V19" s="199" t="s">
         <v>24</v>
       </c>
-      <c r="W19" s="201" t="s">
+      <c r="W19" s="199" t="s">
         <v>25</v>
       </c>
-      <c r="X19" s="201" t="s">
+      <c r="X19" s="199" t="s">
         <v>26</v>
       </c>
-      <c r="Y19" s="201" t="s">
+      <c r="Y19" s="199" t="s">
         <v>27</v>
       </c>
-      <c r="Z19" s="201" t="s">
+      <c r="Z19" s="199" t="s">
         <v>28</v>
       </c>
       <c r="AA19" s="43" t="s">
         <v>29</v>
       </c>
-      <c r="AB19" s="208"/>
-    </row>
-    <row r="20" spans="1:28" ht="36.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="214"/>
-      <c r="B20" s="214"/>
-      <c r="C20" s="211"/>
-      <c r="D20" s="214"/>
-      <c r="E20" s="214"/>
-      <c r="F20" s="237"/>
+      <c r="AB19" s="206"/>
+    </row>
+    <row r="20" spans="1:28" ht="36.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A20" s="212"/>
+      <c r="B20" s="212"/>
+      <c r="C20" s="209"/>
+      <c r="D20" s="212"/>
+      <c r="E20" s="212"/>
+      <c r="F20" s="223"/>
       <c r="G20" s="93" t="s">
         <v>10</v>
       </c>
@@ -11937,17 +11923,17 @@
       <c r="M20" s="18" t="s">
         <v>37</v>
       </c>
-      <c r="O20" s="202"/>
-      <c r="P20" s="202"/>
-      <c r="Q20" s="202"/>
-      <c r="R20" s="202"/>
-      <c r="S20" s="202"/>
+      <c r="O20" s="200"/>
+      <c r="P20" s="200"/>
+      <c r="Q20" s="200"/>
+      <c r="R20" s="200"/>
+      <c r="S20" s="200"/>
       <c r="T20" s="19"/>
-      <c r="V20" s="202"/>
-      <c r="W20" s="202"/>
-      <c r="X20" s="202"/>
-      <c r="Y20" s="202"/>
-      <c r="Z20" s="202"/>
+      <c r="V20" s="200"/>
+      <c r="W20" s="200"/>
+      <c r="X20" s="200"/>
+      <c r="Y20" s="200"/>
+      <c r="Z20" s="200"/>
       <c r="AA20" s="19" t="s">
         <v>20</v>
       </c>
@@ -11955,7 +11941,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="21" spans="1:28" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:28" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A21" s="8">
         <v>1</v>
       </c>
@@ -11968,7 +11954,7 @@
       <c r="D21" s="8" t="s">
         <v>79</v>
       </c>
-      <c r="E21" s="240" t="s">
+      <c r="E21" s="226" t="s">
         <v>102</v>
       </c>
       <c r="F21" s="113">
@@ -12029,7 +12015,7 @@
         <v>3270887.1320000002</v>
       </c>
     </row>
-    <row r="22" spans="1:28" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:28" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A22" s="8">
         <v>2</v>
       </c>
@@ -12042,7 +12028,7 @@
       <c r="D22" s="8" t="s">
         <v>79</v>
       </c>
-      <c r="E22" s="240"/>
+      <c r="E22" s="226"/>
       <c r="F22" s="113">
         <v>45913</v>
       </c>
@@ -12101,7 +12087,7 @@
         <v>3550783.04</v>
       </c>
     </row>
-    <row r="23" spans="1:28" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:28" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A23" s="8">
         <v>3</v>
       </c>
@@ -12114,7 +12100,7 @@
       <c r="D23" s="8" t="s">
         <v>90</v>
       </c>
-      <c r="E23" s="240"/>
+      <c r="E23" s="226"/>
       <c r="F23" s="113">
         <v>45910</v>
       </c>
@@ -12173,7 +12159,7 @@
         <v>253627.36000000002</v>
       </c>
     </row>
-    <row r="24" spans="1:28" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:28" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A24" s="8">
         <v>4</v>
       </c>
@@ -12186,7 +12172,7 @@
       <c r="D24" s="8" t="s">
         <v>90</v>
       </c>
-      <c r="E24" s="240"/>
+      <c r="E24" s="226"/>
       <c r="F24" s="113">
         <v>45927</v>
       </c>
@@ -12245,7 +12231,7 @@
         <v>283519.15600000002</v>
       </c>
     </row>
-    <row r="25" spans="1:28" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:28" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A25" s="8">
         <v>5</v>
       </c>
@@ -12258,7 +12244,7 @@
       <c r="D25" s="8" t="s">
         <v>90</v>
       </c>
-      <c r="E25" s="240"/>
+      <c r="E25" s="226"/>
       <c r="F25" s="113">
         <v>45915</v>
       </c>
@@ -12317,7 +12303,7 @@
         <v>288954.02799999999</v>
       </c>
     </row>
-    <row r="26" spans="1:28" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:28" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A26" s="8">
         <v>6</v>
       </c>
@@ -12391,7 +12377,7 @@
         <v>4491015.8959999997</v>
       </c>
     </row>
-    <row r="27" spans="1:28" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:28" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A27" s="8">
         <v>7</v>
       </c>
@@ -12463,7 +12449,7 @@
         <v>1454734.0720000002</v>
       </c>
     </row>
-    <row r="28" spans="1:28" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:28" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A28" s="8">
         <v>8</v>
       </c>
@@ -12535,7 +12521,7 @@
         <v>292577.27600000001</v>
       </c>
     </row>
-    <row r="29" spans="1:28" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:28" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A29" s="8">
         <v>9</v>
       </c>
@@ -12607,7 +12593,7 @@
         <v>4481051.9639999997</v>
       </c>
     </row>
-    <row r="30" spans="1:28" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:28" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A30" s="8">
         <v>10</v>
       </c>
@@ -12679,7 +12665,7 @@
         <v>2490983</v>
       </c>
     </row>
-    <row r="31" spans="1:28" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:28" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A31" s="8">
         <v>11</v>
       </c>
@@ -12751,7 +12737,7 @@
         <v>244569.24000000002</v>
       </c>
     </row>
-    <row r="32" spans="1:28" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:28" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A32" s="8">
         <v>12</v>
       </c>
@@ -12823,7 +12809,7 @@
         <v>623198.65599999996</v>
       </c>
     </row>
-    <row r="33" spans="1:28" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:28" ht="20.149999999999999" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A33" s="8">
         <v>13</v>
       </c>
@@ -12879,7 +12865,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:28" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:28" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A34" s="9"/>
       <c r="B34" s="10"/>
       <c r="C34" s="124">

</xml_diff>

<commit_message>
Remove outdated Erection output file and update binary files for stringing plans
- Deleted `ErectionCompiled_Output.xlsx` as it is no longer needed.
- Updated `MicroPlanResponsibilities.parquet` and `StringingCompiled_Output.xlsx` to reflect recent changes in data processing.
- Enhanced callback logic in `dashboard/callbacks.py` for improved project data handling and error management.
</commit_message>
<xml_diff>
--- a/Raw Data/Micro Plans/November 2025/Micro Plan - TA-413 Nov'25.xlsx
+++ b/Raw Data/Micro Plans/November 2025/Micro Plan - TA-413 Nov'25.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kaushikb\Documents\Work\Git\Office-work-\Raw Data\Micro Plans\November 2025\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F4D9C61-9FC6-4092-B033-11C8089F33F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA0F693C-B2D8-4F15-8922-8D9FA3D17654}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="757" firstSheet="2" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="447" uniqueCount="231">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="450" uniqueCount="233">
   <si>
     <t>Project Code</t>
   </si>
@@ -742,6 +742,12 @@
   </si>
   <si>
     <t>7/0</t>
+  </si>
+  <si>
+    <t>6/0</t>
+  </si>
+  <si>
+    <t>5/0</t>
   </si>
 </sst>
 </file>
@@ -2173,69 +2179,72 @@
     <xf numFmtId="15" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -2263,6 +2272,9 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -2271,12 +2283,6 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="172">
@@ -6369,137 +6375,137 @@
       <c r="F17" s="6"/>
     </row>
     <row r="18" spans="1:33" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A18" s="211" t="s">
+      <c r="A18" s="197" t="s">
         <v>4</v>
       </c>
-      <c r="B18" s="211" t="s">
+      <c r="B18" s="197" t="s">
         <v>5</v>
       </c>
-      <c r="C18" s="207" t="s">
+      <c r="C18" s="194" t="s">
         <v>6</v>
       </c>
-      <c r="D18" s="211" t="s">
+      <c r="D18" s="197" t="s">
         <v>7</v>
       </c>
-      <c r="E18" s="207" t="s">
+      <c r="E18" s="194" t="s">
         <v>16</v>
       </c>
-      <c r="F18" s="207" t="s">
+      <c r="F18" s="194" t="s">
         <v>17</v>
       </c>
-      <c r="G18" s="211" t="s">
+      <c r="G18" s="197" t="s">
         <v>8</v>
       </c>
-      <c r="H18" s="198" t="s">
+      <c r="H18" s="209" t="s">
         <v>18</v>
       </c>
-      <c r="I18" s="198"/>
-      <c r="J18" s="198"/>
-      <c r="K18" s="198"/>
-      <c r="L18" s="198"/>
-      <c r="M18" s="198"/>
-      <c r="N18" s="198"/>
-      <c r="O18" s="198"/>
-      <c r="P18" s="201" t="s">
+      <c r="I18" s="209"/>
+      <c r="J18" s="209"/>
+      <c r="K18" s="209"/>
+      <c r="L18" s="209"/>
+      <c r="M18" s="209"/>
+      <c r="N18" s="209"/>
+      <c r="O18" s="209"/>
+      <c r="P18" s="202" t="s">
         <v>19</v>
       </c>
-      <c r="R18" s="207" t="s">
+      <c r="R18" s="194" t="s">
         <v>36</v>
       </c>
-      <c r="T18" s="202" t="s">
+      <c r="T18" s="203" t="s">
         <v>31</v>
       </c>
-      <c r="U18" s="203"/>
-      <c r="V18" s="203"/>
-      <c r="W18" s="203"/>
-      <c r="X18" s="203"/>
-      <c r="Y18" s="204"/>
-      <c r="AA18" s="202" t="s">
+      <c r="U18" s="204"/>
+      <c r="V18" s="204"/>
+      <c r="W18" s="204"/>
+      <c r="X18" s="204"/>
+      <c r="Y18" s="205"/>
+      <c r="AA18" s="203" t="s">
         <v>30</v>
       </c>
-      <c r="AB18" s="203"/>
-      <c r="AC18" s="203"/>
-      <c r="AD18" s="203"/>
-      <c r="AE18" s="203"/>
-      <c r="AF18" s="204"/>
-      <c r="AG18" s="205" t="s">
+      <c r="AB18" s="204"/>
+      <c r="AC18" s="204"/>
+      <c r="AD18" s="204"/>
+      <c r="AE18" s="204"/>
+      <c r="AF18" s="205"/>
+      <c r="AG18" s="206" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="19" spans="1:33" ht="21" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A19" s="212"/>
-      <c r="B19" s="212"/>
-      <c r="C19" s="209"/>
-      <c r="D19" s="212"/>
-      <c r="E19" s="209"/>
-      <c r="F19" s="209"/>
-      <c r="G19" s="212"/>
-      <c r="H19" s="197" t="s">
+      <c r="A19" s="198"/>
+      <c r="B19" s="198"/>
+      <c r="C19" s="195"/>
+      <c r="D19" s="198"/>
+      <c r="E19" s="195"/>
+      <c r="F19" s="195"/>
+      <c r="G19" s="198"/>
+      <c r="H19" s="214" t="s">
         <v>9</v>
       </c>
-      <c r="I19" s="197"/>
-      <c r="J19" s="197" t="s">
+      <c r="I19" s="214"/>
+      <c r="J19" s="214" t="s">
         <v>12</v>
       </c>
-      <c r="K19" s="197"/>
-      <c r="L19" s="197" t="s">
+      <c r="K19" s="214"/>
+      <c r="L19" s="214" t="s">
         <v>13</v>
       </c>
-      <c r="M19" s="197"/>
-      <c r="N19" s="195" t="s">
+      <c r="M19" s="214"/>
+      <c r="N19" s="210" t="s">
         <v>15</v>
       </c>
-      <c r="O19" s="195" t="s">
+      <c r="O19" s="210" t="s">
         <v>14</v>
       </c>
-      <c r="P19" s="201"/>
+      <c r="P19" s="202"/>
       <c r="R19" s="208"/>
-      <c r="T19" s="199" t="s">
+      <c r="T19" s="200" t="s">
         <v>24</v>
       </c>
-      <c r="U19" s="199" t="s">
+      <c r="U19" s="200" t="s">
         <v>25</v>
       </c>
-      <c r="V19" s="199" t="s">
+      <c r="V19" s="200" t="s">
         <v>26</v>
       </c>
-      <c r="W19" s="199" t="s">
+      <c r="W19" s="200" t="s">
         <v>27</v>
       </c>
-      <c r="X19" s="199" t="s">
+      <c r="X19" s="200" t="s">
         <v>28</v>
       </c>
       <c r="Y19" s="43" t="s">
         <v>29</v>
       </c>
-      <c r="AA19" s="199" t="s">
+      <c r="AA19" s="200" t="s">
         <v>24</v>
       </c>
-      <c r="AB19" s="199" t="s">
+      <c r="AB19" s="200" t="s">
         <v>25</v>
       </c>
-      <c r="AC19" s="199" t="s">
+      <c r="AC19" s="200" t="s">
         <v>26</v>
       </c>
-      <c r="AD19" s="199" t="s">
+      <c r="AD19" s="200" t="s">
         <v>27</v>
       </c>
-      <c r="AE19" s="199" t="s">
+      <c r="AE19" s="200" t="s">
         <v>28</v>
       </c>
       <c r="AF19" s="43" t="s">
         <v>29</v>
       </c>
-      <c r="AG19" s="206"/>
+      <c r="AG19" s="207"/>
     </row>
     <row r="20" spans="1:33" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A20" s="213"/>
-      <c r="B20" s="212"/>
-      <c r="C20" s="209"/>
-      <c r="D20" s="212"/>
-      <c r="E20" s="210"/>
-      <c r="F20" s="210"/>
-      <c r="G20" s="212"/>
+      <c r="A20" s="199"/>
+      <c r="B20" s="198"/>
+      <c r="C20" s="195"/>
+      <c r="D20" s="198"/>
+      <c r="E20" s="196"/>
+      <c r="F20" s="196"/>
+      <c r="G20" s="198"/>
       <c r="H20" s="93" t="s">
         <v>10</v>
       </c>
@@ -6518,25 +6524,25 @@
       <c r="M20" s="93" t="s">
         <v>11</v>
       </c>
-      <c r="N20" s="196"/>
-      <c r="O20" s="196"/>
+      <c r="N20" s="211"/>
+      <c r="O20" s="211"/>
       <c r="P20" s="44" t="s">
         <v>50</v>
       </c>
       <c r="R20" s="18" t="s">
         <v>37</v>
       </c>
-      <c r="T20" s="200"/>
-      <c r="U20" s="200"/>
-      <c r="V20" s="200"/>
-      <c r="W20" s="200"/>
-      <c r="X20" s="200"/>
+      <c r="T20" s="201"/>
+      <c r="U20" s="201"/>
+      <c r="V20" s="201"/>
+      <c r="W20" s="201"/>
+      <c r="X20" s="201"/>
       <c r="Y20" s="19"/>
-      <c r="AA20" s="200"/>
-      <c r="AB20" s="200"/>
-      <c r="AC20" s="200"/>
-      <c r="AD20" s="200"/>
-      <c r="AE20" s="200"/>
+      <c r="AA20" s="201"/>
+      <c r="AB20" s="201"/>
+      <c r="AC20" s="201"/>
+      <c r="AD20" s="201"/>
+      <c r="AE20" s="201"/>
       <c r="AF20" s="19" t="s">
         <v>50</v>
       </c>
@@ -6807,7 +6813,7 @@
       <c r="D25" s="85"/>
       <c r="E25" s="100"/>
       <c r="F25" s="8"/>
-      <c r="G25" s="193"/>
+      <c r="G25" s="212"/>
       <c r="H25" s="98"/>
       <c r="I25" s="98"/>
       <c r="J25" s="98"/>
@@ -6865,7 +6871,7 @@
       <c r="D26" s="8"/>
       <c r="E26" s="101"/>
       <c r="F26" s="96"/>
-      <c r="G26" s="194"/>
+      <c r="G26" s="213"/>
       <c r="H26" s="98"/>
       <c r="I26" s="98"/>
       <c r="J26" s="98"/>
@@ -7220,13 +7226,16 @@
     <filterColumn colId="13" showButton="0"/>
   </autoFilter>
   <mergeCells count="29">
-    <mergeCell ref="F18:F20"/>
-    <mergeCell ref="G18:G20"/>
-    <mergeCell ref="A18:A20"/>
-    <mergeCell ref="B18:B20"/>
-    <mergeCell ref="C18:C20"/>
-    <mergeCell ref="D18:D20"/>
-    <mergeCell ref="E18:E20"/>
+    <mergeCell ref="G25:G26"/>
+    <mergeCell ref="O19:O20"/>
+    <mergeCell ref="H19:I19"/>
+    <mergeCell ref="J19:K19"/>
+    <mergeCell ref="L19:M19"/>
+    <mergeCell ref="H18:O18"/>
+    <mergeCell ref="N19:N20"/>
+    <mergeCell ref="U19:U20"/>
+    <mergeCell ref="V19:V20"/>
+    <mergeCell ref="W19:W20"/>
     <mergeCell ref="X19:X20"/>
     <mergeCell ref="P18:P19"/>
     <mergeCell ref="AA18:AF18"/>
@@ -7239,16 +7248,13 @@
     <mergeCell ref="R18:R19"/>
     <mergeCell ref="T18:Y18"/>
     <mergeCell ref="T19:T20"/>
-    <mergeCell ref="H18:O18"/>
-    <mergeCell ref="N19:N20"/>
-    <mergeCell ref="U19:U20"/>
-    <mergeCell ref="V19:V20"/>
-    <mergeCell ref="W19:W20"/>
-    <mergeCell ref="G25:G26"/>
-    <mergeCell ref="O19:O20"/>
-    <mergeCell ref="H19:I19"/>
-    <mergeCell ref="J19:K19"/>
-    <mergeCell ref="L19:M19"/>
+    <mergeCell ref="F18:F20"/>
+    <mergeCell ref="G18:G20"/>
+    <mergeCell ref="A18:A20"/>
+    <mergeCell ref="B18:B20"/>
+    <mergeCell ref="C18:C20"/>
+    <mergeCell ref="D18:D20"/>
+    <mergeCell ref="E18:E20"/>
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="B21">
@@ -7519,7 +7525,7 @@
       <c r="Q4" s="70">
         <v>0</v>
       </c>
-      <c r="R4" s="214" t="s">
+      <c r="R4" s="215" t="s">
         <v>75</v>
       </c>
     </row>
@@ -7562,14 +7568,14 @@
       <c r="Q5" s="70">
         <v>0</v>
       </c>
-      <c r="R5" s="215"/>
+      <c r="R5" s="216"/>
     </row>
     <row r="6" spans="2:18" s="75" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="B6" s="216" t="s">
+      <c r="B6" s="217" t="s">
         <v>29</v>
       </c>
-      <c r="C6" s="217"/>
-      <c r="D6" s="218"/>
+      <c r="C6" s="218"/>
+      <c r="D6" s="219"/>
       <c r="E6" s="73">
         <v>160</v>
       </c>
@@ -11088,64 +11094,64 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:16" x14ac:dyDescent="0.35">
-      <c r="B1" s="219" t="s">
+      <c r="B1" s="220" t="s">
         <v>198</v>
       </c>
-      <c r="C1" s="219"/>
-      <c r="D1" s="219"/>
-      <c r="E1" s="219"/>
-      <c r="F1" s="219"/>
-      <c r="G1" s="219"/>
-      <c r="H1" s="219"/>
-      <c r="I1" s="219"/>
-      <c r="J1" s="219"/>
-      <c r="K1" s="219"/>
-      <c r="L1" s="219"/>
+      <c r="C1" s="220"/>
+      <c r="D1" s="220"/>
+      <c r="E1" s="220"/>
+      <c r="F1" s="220"/>
+      <c r="G1" s="220"/>
+      <c r="H1" s="220"/>
+      <c r="I1" s="220"/>
+      <c r="J1" s="220"/>
+      <c r="K1" s="220"/>
+      <c r="L1" s="220"/>
     </row>
     <row r="2" spans="2:16" x14ac:dyDescent="0.35">
-      <c r="B2" s="220" t="s">
+      <c r="B2" s="221" t="s">
         <v>199</v>
       </c>
-      <c r="C2" s="220"/>
-      <c r="D2" s="220"/>
-      <c r="E2" s="220"/>
-      <c r="F2" s="220"/>
-      <c r="G2" s="220"/>
-      <c r="H2" s="220"/>
-      <c r="I2" s="220"/>
-      <c r="J2" s="220"/>
-      <c r="K2" s="220"/>
-      <c r="L2" s="220"/>
+      <c r="C2" s="221"/>
+      <c r="D2" s="221"/>
+      <c r="E2" s="221"/>
+      <c r="F2" s="221"/>
+      <c r="G2" s="221"/>
+      <c r="H2" s="221"/>
+      <c r="I2" s="221"/>
+      <c r="J2" s="221"/>
+      <c r="K2" s="221"/>
+      <c r="L2" s="221"/>
     </row>
     <row r="3" spans="2:16" x14ac:dyDescent="0.35">
-      <c r="B3" s="221" t="s">
+      <c r="B3" s="222" t="s">
         <v>200</v>
       </c>
-      <c r="C3" s="221"/>
-      <c r="D3" s="221"/>
-      <c r="E3" s="221"/>
-      <c r="F3" s="221"/>
-      <c r="G3" s="221"/>
-      <c r="H3" s="221"/>
-      <c r="I3" s="221"/>
-      <c r="J3" s="221"/>
-      <c r="K3" s="221"/>
-      <c r="L3" s="221"/>
+      <c r="C3" s="222"/>
+      <c r="D3" s="222"/>
+      <c r="E3" s="222"/>
+      <c r="F3" s="222"/>
+      <c r="G3" s="222"/>
+      <c r="H3" s="222"/>
+      <c r="I3" s="222"/>
+      <c r="J3" s="222"/>
+      <c r="K3" s="222"/>
+      <c r="L3" s="222"/>
     </row>
     <row r="4" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B4" s="222" t="s">
+      <c r="B4" s="223" t="s">
         <v>201</v>
       </c>
-      <c r="C4" s="222"/>
-      <c r="D4" s="222"/>
-      <c r="E4" s="222"/>
-      <c r="F4" s="222"/>
-      <c r="G4" s="222"/>
-      <c r="H4" s="222"/>
-      <c r="I4" s="222"/>
-      <c r="J4" s="222"/>
-      <c r="K4" s="222"/>
-      <c r="L4" s="222"/>
+      <c r="C4" s="223"/>
+      <c r="D4" s="223"/>
+      <c r="E4" s="223"/>
+      <c r="F4" s="223"/>
+      <c r="G4" s="223"/>
+      <c r="H4" s="223"/>
+      <c r="I4" s="223"/>
+      <c r="J4" s="223"/>
+      <c r="K4" s="223"/>
+      <c r="L4" s="223"/>
     </row>
     <row r="5" spans="2:16" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B5" s="186" t="s">
@@ -11212,10 +11218,10 @@
       <c r="B7" s="191">
         <v>1</v>
       </c>
-      <c r="C7" s="191">
-        <v>6</v>
-      </c>
-      <c r="D7" s="227" t="s">
+      <c r="C7" s="193" t="s">
+        <v>231</v>
+      </c>
+      <c r="D7" s="193" t="s">
         <v>230</v>
       </c>
       <c r="E7" s="191">
@@ -11257,8 +11263,8 @@
       <c r="B8" s="191">
         <v>2</v>
       </c>
-      <c r="C8" s="191">
-        <v>5</v>
+      <c r="C8" s="193" t="s">
+        <v>232</v>
       </c>
       <c r="D8" s="191" t="s">
         <v>225</v>
@@ -11305,8 +11311,8 @@
       <c r="C9" s="191" t="s">
         <v>225</v>
       </c>
-      <c r="D9" s="191">
-        <v>6</v>
+      <c r="D9" s="193" t="s">
+        <v>231</v>
       </c>
       <c r="E9" s="191">
         <v>419.48</v>
@@ -11793,118 +11799,118 @@
       <c r="F17" s="6"/>
     </row>
     <row r="18" spans="1:28" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A18" s="211" t="s">
+      <c r="A18" s="197" t="s">
         <v>4</v>
       </c>
-      <c r="B18" s="211" t="s">
+      <c r="B18" s="197" t="s">
         <v>42</v>
       </c>
-      <c r="C18" s="207" t="s">
+      <c r="C18" s="194" t="s">
         <v>47</v>
       </c>
-      <c r="D18" s="207" t="s">
+      <c r="D18" s="194" t="s">
         <v>43</v>
       </c>
-      <c r="E18" s="211" t="s">
+      <c r="E18" s="197" t="s">
         <v>8</v>
       </c>
-      <c r="F18" s="198" t="s">
+      <c r="F18" s="209" t="s">
         <v>18</v>
       </c>
-      <c r="G18" s="198"/>
-      <c r="H18" s="198"/>
-      <c r="I18" s="198"/>
-      <c r="J18" s="198"/>
-      <c r="K18" s="201" t="s">
+      <c r="G18" s="209"/>
+      <c r="H18" s="209"/>
+      <c r="I18" s="209"/>
+      <c r="J18" s="209"/>
+      <c r="K18" s="202" t="s">
         <v>19</v>
       </c>
-      <c r="M18" s="207" t="s">
+      <c r="M18" s="194" t="s">
         <v>36</v>
       </c>
-      <c r="O18" s="202" t="s">
+      <c r="O18" s="203" t="s">
         <v>31</v>
       </c>
-      <c r="P18" s="203"/>
-      <c r="Q18" s="203"/>
-      <c r="R18" s="203"/>
-      <c r="S18" s="203"/>
-      <c r="T18" s="204"/>
-      <c r="V18" s="202" t="s">
+      <c r="P18" s="204"/>
+      <c r="Q18" s="204"/>
+      <c r="R18" s="204"/>
+      <c r="S18" s="204"/>
+      <c r="T18" s="205"/>
+      <c r="V18" s="203" t="s">
         <v>30</v>
       </c>
-      <c r="W18" s="203"/>
-      <c r="X18" s="203"/>
-      <c r="Y18" s="203"/>
-      <c r="Z18" s="203"/>
-      <c r="AA18" s="204"/>
-      <c r="AB18" s="205" t="s">
+      <c r="W18" s="204"/>
+      <c r="X18" s="204"/>
+      <c r="Y18" s="204"/>
+      <c r="Z18" s="204"/>
+      <c r="AA18" s="205"/>
+      <c r="AB18" s="206" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="19" spans="1:28" ht="21" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A19" s="212"/>
-      <c r="B19" s="212"/>
-      <c r="C19" s="209"/>
-      <c r="D19" s="212"/>
-      <c r="E19" s="212"/>
-      <c r="F19" s="223" t="s">
+      <c r="A19" s="198"/>
+      <c r="B19" s="198"/>
+      <c r="C19" s="195"/>
+      <c r="D19" s="198"/>
+      <c r="E19" s="198"/>
+      <c r="F19" s="225" t="s">
         <v>40</v>
       </c>
-      <c r="G19" s="224" t="s">
+      <c r="G19" s="226" t="s">
         <v>44</v>
       </c>
-      <c r="H19" s="225"/>
-      <c r="I19" s="224" t="s">
+      <c r="H19" s="227"/>
+      <c r="I19" s="226" t="s">
         <v>45</v>
       </c>
-      <c r="J19" s="225"/>
-      <c r="K19" s="201"/>
+      <c r="J19" s="227"/>
+      <c r="K19" s="202"/>
       <c r="M19" s="208"/>
-      <c r="O19" s="199" t="s">
+      <c r="O19" s="200" t="s">
         <v>24</v>
       </c>
-      <c r="P19" s="199" t="s">
+      <c r="P19" s="200" t="s">
         <v>25</v>
       </c>
-      <c r="Q19" s="199" t="s">
+      <c r="Q19" s="200" t="s">
         <v>26</v>
       </c>
-      <c r="R19" s="199" t="s">
+      <c r="R19" s="200" t="s">
         <v>27</v>
       </c>
-      <c r="S19" s="199" t="s">
+      <c r="S19" s="200" t="s">
         <v>28</v>
       </c>
       <c r="T19" s="43" t="s">
         <v>29</v>
       </c>
-      <c r="V19" s="199" t="s">
+      <c r="V19" s="200" t="s">
         <v>24</v>
       </c>
-      <c r="W19" s="199" t="s">
+      <c r="W19" s="200" t="s">
         <v>25</v>
       </c>
-      <c r="X19" s="199" t="s">
+      <c r="X19" s="200" t="s">
         <v>26</v>
       </c>
-      <c r="Y19" s="199" t="s">
+      <c r="Y19" s="200" t="s">
         <v>27</v>
       </c>
-      <c r="Z19" s="199" t="s">
+      <c r="Z19" s="200" t="s">
         <v>28</v>
       </c>
       <c r="AA19" s="43" t="s">
         <v>29</v>
       </c>
-      <c r="AB19" s="206"/>
+      <c r="AB19" s="207"/>
     </row>
     <row r="20" spans="1:28" ht="36.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A20" s="212"/>
-      <c r="B20" s="212"/>
-      <c r="C20" s="209"/>
-      <c r="D20" s="212"/>
-      <c r="E20" s="212"/>
-      <c r="F20" s="223"/>
+      <c r="A20" s="198"/>
+      <c r="B20" s="198"/>
+      <c r="C20" s="195"/>
+      <c r="D20" s="198"/>
+      <c r="E20" s="198"/>
+      <c r="F20" s="225"/>
       <c r="G20" s="93" t="s">
         <v>10</v>
       </c>
@@ -11923,17 +11929,17 @@
       <c r="M20" s="18" t="s">
         <v>37</v>
       </c>
-      <c r="O20" s="200"/>
-      <c r="P20" s="200"/>
-      <c r="Q20" s="200"/>
-      <c r="R20" s="200"/>
-      <c r="S20" s="200"/>
+      <c r="O20" s="201"/>
+      <c r="P20" s="201"/>
+      <c r="Q20" s="201"/>
+      <c r="R20" s="201"/>
+      <c r="S20" s="201"/>
       <c r="T20" s="19"/>
-      <c r="V20" s="200"/>
-      <c r="W20" s="200"/>
-      <c r="X20" s="200"/>
-      <c r="Y20" s="200"/>
-      <c r="Z20" s="200"/>
+      <c r="V20" s="201"/>
+      <c r="W20" s="201"/>
+      <c r="X20" s="201"/>
+      <c r="Y20" s="201"/>
+      <c r="Z20" s="201"/>
       <c r="AA20" s="19" t="s">
         <v>20</v>
       </c>
@@ -11954,7 +11960,7 @@
       <c r="D21" s="8" t="s">
         <v>79</v>
       </c>
-      <c r="E21" s="226" t="s">
+      <c r="E21" s="224" t="s">
         <v>102</v>
       </c>
       <c r="F21" s="113">
@@ -12028,7 +12034,7 @@
       <c r="D22" s="8" t="s">
         <v>79</v>
       </c>
-      <c r="E22" s="226"/>
+      <c r="E22" s="224"/>
       <c r="F22" s="113">
         <v>45913</v>
       </c>
@@ -12100,7 +12106,7 @@
       <c r="D23" s="8" t="s">
         <v>90</v>
       </c>
-      <c r="E23" s="226"/>
+      <c r="E23" s="224"/>
       <c r="F23" s="113">
         <v>45910</v>
       </c>
@@ -12172,7 +12178,7 @@
       <c r="D24" s="8" t="s">
         <v>90</v>
       </c>
-      <c r="E24" s="226"/>
+      <c r="E24" s="224"/>
       <c r="F24" s="113">
         <v>45927</v>
       </c>
@@ -12244,7 +12250,7 @@
       <c r="D25" s="8" t="s">
         <v>90</v>
       </c>
-      <c r="E25" s="226"/>
+      <c r="E25" s="224"/>
       <c r="F25" s="113">
         <v>45915</v>
       </c>
@@ -12939,18 +12945,6 @@
     </row>
   </sheetData>
   <mergeCells count="25">
-    <mergeCell ref="E21:E25"/>
-    <mergeCell ref="W19:W20"/>
-    <mergeCell ref="K18:K19"/>
-    <mergeCell ref="M18:M19"/>
-    <mergeCell ref="O18:T18"/>
-    <mergeCell ref="V18:AA18"/>
-    <mergeCell ref="V19:V20"/>
-    <mergeCell ref="A18:A20"/>
-    <mergeCell ref="B18:B20"/>
-    <mergeCell ref="C18:C20"/>
-    <mergeCell ref="D18:D20"/>
-    <mergeCell ref="E18:E20"/>
     <mergeCell ref="AB18:AB19"/>
     <mergeCell ref="F19:F20"/>
     <mergeCell ref="G19:H19"/>
@@ -12964,6 +12958,18 @@
     <mergeCell ref="Q19:Q20"/>
     <mergeCell ref="R19:R20"/>
     <mergeCell ref="S19:S20"/>
+    <mergeCell ref="A18:A20"/>
+    <mergeCell ref="B18:B20"/>
+    <mergeCell ref="C18:C20"/>
+    <mergeCell ref="D18:D20"/>
+    <mergeCell ref="E18:E20"/>
+    <mergeCell ref="E21:E25"/>
+    <mergeCell ref="W19:W20"/>
+    <mergeCell ref="K18:K19"/>
+    <mergeCell ref="M18:M19"/>
+    <mergeCell ref="O18:T18"/>
+    <mergeCell ref="V18:AA18"/>
+    <mergeCell ref="V19:V20"/>
   </mergeCells>
   <conditionalFormatting sqref="C26:C27">
     <cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="4DT6">

</xml_diff>